<commit_message>
Excel 2026-09-25: rebuild dxl-metrics.xlsx from the three fresh rollups
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-09-24 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-09-25 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">80 dòng × 7 chỉ số · 2026-07-05 → 2026-09-22</t>
+    <t xml:space="preserve">81 dòng × 7 chỉ số · 2026-07-05 → 2026-09-23</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">44 dòng × 14 chỉ số · 2026-07-23 → 2026-09-24</t>
+    <t xml:space="preserve">45 dòng × 14 chỉ số · 2026-07-23 → 2026-09-25</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">44 dòng × 14 chỉ số · 2026-06-30 → 2026-09-24</t>
+    <t xml:space="preserve">45 dòng × 14 chỉ số · 2026-06-30 → 2026-09-25</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">41 dòng × 11 chỉ số · 2026-07-27 → 2026-09-24</t>
+    <t xml:space="preserve">42 dòng × 11 chỉ số · 2026-07-27 → 2026-09-25</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 80 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 81 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 44 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 45 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 44 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 45 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 41 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 42 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -978,7 +978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3130,6 +3130,32 @@
       </c>
       <c r="H85" s="16" t="n">
         <v>29</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="15" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B86" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C86" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" s="16" t="n">
+        <v>187</v>
+      </c>
+      <c r="E86" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="F86" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G86" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="H86" s="16" t="n">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -3148,7 +3174,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5330,6 +5356,53 @@
       </c>
       <c r="O49" s="16" t="n">
         <v>634</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="15" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <v>135</v>
+      </c>
+      <c r="D50" s="16" t="n">
+        <v>4560</v>
+      </c>
+      <c r="E50" s="16" t="n">
+        <v>486</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G50" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="H50" s="16" t="n">
+        <v>86</v>
+      </c>
+      <c r="I50" s="16" t="n">
+        <v>2422</v>
+      </c>
+      <c r="J50" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K50" s="16" t="n">
+        <v>1328</v>
+      </c>
+      <c r="L50" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="M50" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="N50" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O50" s="16" t="n">
+        <v>635</v>
       </c>
     </row>
   </sheetData>
@@ -5348,7 +5421,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7434,6 +7507,53 @@
       </c>
       <c r="O49" s="16" t="n">
         <v>328</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="15" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <v>699</v>
+      </c>
+      <c r="D50" s="16" t="n">
+        <v>663</v>
+      </c>
+      <c r="E50" s="19" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" s="16" t="n">
+        <v>584</v>
+      </c>
+      <c r="H50" s="16" t="n">
+        <v>399</v>
+      </c>
+      <c r="I50" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="J50" s="19" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="K50" s="16" t="n">
+        <v>1034</v>
+      </c>
+      <c r="L50" s="19" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="M50" s="16" t="n">
+        <v>86</v>
+      </c>
+      <c r="N50" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O50" s="16" t="n">
+        <v>336</v>
       </c>
     </row>
   </sheetData>
@@ -7452,7 +7572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8968,6 +9088,44 @@
       </c>
       <c r="L46" s="16" t="n">
         <v>239199</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="15" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B47" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="C47" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="D47" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="E47" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F47" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G47" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H47" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I47" s="16" t="n">
+        <v>88</v>
+      </c>
+      <c r="J47" s="16" t="n">
+        <v>336</v>
+      </c>
+      <c r="K47" s="16" t="n">
+        <v>274</v>
+      </c>
+      <c r="L47" s="16" t="n">
+        <v>239208</v>
       </c>
     </row>
   </sheetData>
@@ -9032,16 +9190,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>111</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>118</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9049,16 +9207,16 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>341</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>345</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9066,16 +9224,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>3782</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>3969</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9083,16 +9241,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>349</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>380</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9100,16 +9258,16 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>11</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9117,16 +9275,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>140</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>147</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9134,16 +9292,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H85,'Social — theo ngày'!$A$6:$A$85,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$85,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2112</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2157</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9178,7 +9336,7 @@
         <v>115</v>
       </c>
       <c r="D17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B49</f>
+        <f aca="false">'Social — 28 ngày'!B50</f>
         <v>116</v>
       </c>
     </row>
@@ -9195,8 +9353,8 @@
         <v>184</v>
       </c>
       <c r="D18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C49</f>
-        <v>137</v>
+        <f aca="false">'Social — 28 ngày'!C50</f>
+        <v>135</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9212,8 +9370,8 @@
         <v>4735</v>
       </c>
       <c r="D19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D49</f>
-        <v>4514</v>
+        <f aca="false">'Social — 28 ngày'!D50</f>
+        <v>4560</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9229,8 +9387,8 @@
         <v>280</v>
       </c>
       <c r="D20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E49</f>
-        <v>455</v>
+        <f aca="false">'Social — 28 ngày'!E50</f>
+        <v>486</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9246,7 +9404,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F49</f>
+        <f aca="false">'Social — 28 ngày'!F50</f>
         <v>49</v>
       </c>
     </row>
@@ -9263,8 +9421,8 @@
         <v>68</v>
       </c>
       <c r="D22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G49</f>
-        <v>13</v>
+        <f aca="false">'Social — 28 ngày'!G50</f>
+        <v>15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9280,7 +9438,7 @@
         <v>275</v>
       </c>
       <c r="D23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H49</f>
+        <f aca="false">'Social — 28 ngày'!H50</f>
         <v>86</v>
       </c>
     </row>
@@ -9297,8 +9455,8 @@
         <v>1039</v>
       </c>
       <c r="D24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I49</f>
-        <v>2485</v>
+        <f aca="false">'Social — 28 ngày'!I50</f>
+        <v>2422</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9314,7 +9472,7 @@
         <v>100</v>
       </c>
       <c r="D25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J49</f>
+        <f aca="false">'Social — 28 ngày'!J50</f>
         <v>102</v>
       </c>
     </row>
@@ -9331,8 +9489,8 @@
         <v>1691</v>
       </c>
       <c r="D26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K49</f>
-        <v>1320</v>
+        <f aca="false">'Social — 28 ngày'!K50</f>
+        <v>1328</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9348,8 +9506,8 @@
         <v>127</v>
       </c>
       <c r="D27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L49</f>
-        <v>36</v>
+        <f aca="false">'Social — 28 ngày'!L50</f>
+        <v>33</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9365,8 +9523,8 @@
         <v>86</v>
       </c>
       <c r="D28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M49</f>
-        <v>58</v>
+        <f aca="false">'Social — 28 ngày'!M50</f>
+        <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9382,7 +9540,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N49</f>
+        <f aca="false">'Social — 28 ngày'!N50</f>
         <v>4</v>
       </c>
     </row>
@@ -9399,8 +9557,8 @@
         <v>59</v>
       </c>
       <c r="D30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O49</f>
-        <v>634</v>
+        <f aca="false">'Social — 28 ngày'!O50</f>
+        <v>635</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9442,7 +9600,7 @@
         <v>21</v>
       </c>
       <c r="E34" s="24" t="n">
-        <f aca="false">SEO!B49</f>
+        <f aca="false">SEO!B50</f>
         <v>12</v>
       </c>
     </row>
@@ -9463,8 +9621,8 @@
         <v>364</v>
       </c>
       <c r="E35" s="24" t="n">
-        <f aca="false">SEO!C49</f>
-        <v>697</v>
+        <f aca="false">SEO!C50</f>
+        <v>699</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9484,8 +9642,8 @@
         <v>349</v>
       </c>
       <c r="E36" s="24" t="n">
-        <f aca="false">SEO!D49</f>
-        <v>661</v>
+        <f aca="false">SEO!D50</f>
+        <v>663</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9505,8 +9663,8 @@
         <v>42.93</v>
       </c>
       <c r="E37" s="24" t="n">
-        <f aca="false">SEO!E49</f>
-        <v>36.87</v>
+        <f aca="false">SEO!E50</f>
+        <v>33.9</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9526,8 +9684,8 @@
         <v>7</v>
       </c>
       <c r="E38" s="24" t="n">
-        <f aca="false">SEO!F49</f>
-        <v>1</v>
+        <f aca="false">SEO!F50</f>
+        <v>3</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9547,8 +9705,8 @@
         <v>375</v>
       </c>
       <c r="E39" s="24" t="n">
-        <f aca="false">SEO!G49</f>
-        <v>575</v>
+        <f aca="false">SEO!G50</f>
+        <v>584</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9568,8 +9726,8 @@
         <v>204</v>
       </c>
       <c r="E40" s="24" t="n">
-        <f aca="false">SEO!H49</f>
-        <v>383</v>
+        <f aca="false">SEO!H50</f>
+        <v>399</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,7 +9747,7 @@
         <v>67</v>
       </c>
       <c r="E41" s="24" t="n">
-        <f aca="false">SEO!I49</f>
+        <f aca="false">SEO!I50</f>
         <v>34</v>
       </c>
     </row>
@@ -9610,8 +9768,8 @@
         <v>3.8</v>
       </c>
       <c r="E42" s="24" t="n">
-        <f aca="false">SEO!J49</f>
-        <v>3.1</v>
+        <f aca="false">SEO!J50</f>
+        <v>3.3</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9631,8 +9789,8 @@
         <v>1757</v>
       </c>
       <c r="E43" s="24" t="n">
-        <f aca="false">SEO!K49</f>
-        <v>1087</v>
+        <f aca="false">SEO!K50</f>
+        <v>1034</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9652,8 +9810,8 @@
         <v>29.4</v>
       </c>
       <c r="E44" s="24" t="n">
-        <f aca="false">SEO!L49</f>
-        <v>31.1</v>
+        <f aca="false">SEO!L50</f>
+        <v>29.1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9673,8 +9831,8 @@
         <v>151</v>
       </c>
       <c r="E45" s="24" t="n">
-        <f aca="false">SEO!M49</f>
-        <v>95</v>
+        <f aca="false">SEO!M50</f>
+        <v>86</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9694,7 +9852,7 @@
         <v>95</v>
       </c>
       <c r="E46" s="24" t="n">
-        <f aca="false">SEO!N49</f>
+        <f aca="false">SEO!N50</f>
         <v>119</v>
       </c>
     </row>
@@ -9715,8 +9873,8 @@
         <v>1022</v>
       </c>
       <c r="E47" s="24" t="n">
-        <f aca="false">SEO!O49</f>
-        <v>328</v>
+        <f aca="false">SEO!O50</f>
+        <v>336</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9751,7 +9909,7 @@
         <v>88</v>
       </c>
       <c r="D51" s="24" t="n">
-        <f aca="false">Audit!B46</f>
+        <f aca="false">Audit!B47</f>
         <v>92</v>
       </c>
     </row>
@@ -9768,8 +9926,8 @@
         <v>97</v>
       </c>
       <c r="D52" s="24" t="n">
-        <f aca="false">Audit!C46</f>
-        <v>92</v>
+        <f aca="false">Audit!C47</f>
+        <v>93</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9785,7 +9943,7 @@
         <v>92</v>
       </c>
       <c r="D53" s="24" t="n">
-        <f aca="false">Audit!D46</f>
+        <f aca="false">Audit!D47</f>
         <v>93</v>
       </c>
     </row>
@@ -9802,7 +9960,7 @@
         <v>91</v>
       </c>
       <c r="D54" s="24" t="n">
-        <f aca="false">Audit!E46</f>
+        <f aca="false">Audit!E47</f>
         <v>92</v>
       </c>
     </row>
@@ -9819,7 +9977,7 @@
         <v>91</v>
       </c>
       <c r="D55" s="24" t="n">
-        <f aca="false">Audit!F46</f>
+        <f aca="false">Audit!F47</f>
         <v>118</v>
       </c>
     </row>
@@ -9836,8 +9994,8 @@
         <v>88</v>
       </c>
       <c r="D56" s="24" t="n">
-        <f aca="false">Audit!G46</f>
-        <v>99</v>
+        <f aca="false">Audit!G47</f>
+        <v>98</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9853,7 +10011,7 @@
         <v>92</v>
       </c>
       <c r="D57" s="24" t="n">
-        <f aca="false">Audit!H46</f>
+        <f aca="false">Audit!H47</f>
         <v>119</v>
       </c>
     </row>
@@ -9870,7 +10028,7 @@
         <v>96</v>
       </c>
       <c r="D58" s="24" t="n">
-        <f aca="false">Audit!I46</f>
+        <f aca="false">Audit!I47</f>
         <v>88</v>
       </c>
     </row>
@@ -9887,8 +10045,8 @@
         <v>862</v>
       </c>
       <c r="D59" s="24" t="n">
-        <f aca="false">Audit!J46</f>
-        <v>328</v>
+        <f aca="false">Audit!J47</f>
+        <v>336</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9904,8 +10062,8 @@
         <v>0</v>
       </c>
       <c r="D60" s="24" t="n">
-        <f aca="false">Audit!K46</f>
-        <v>267</v>
+        <f aca="false">Audit!K47</f>
+        <v>274</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9921,8 +10079,8 @@
         <v>0</v>
       </c>
       <c r="D61" s="24" t="n">
-        <f aca="false">Audit!L46</f>
-        <v>239199</v>
+        <f aca="false">Audit!L47</f>
+        <v>239208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel 2026-09-26: rebuild dxl-metrics.xlsx from the three fresh rollups (recalc 152 formulas, 0 errors)
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-09-25 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-09-26 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">81 dòng × 7 chỉ số · 2026-07-05 → 2026-09-23</t>
+    <t xml:space="preserve">82 dòng × 7 chỉ số · 2026-07-05 → 2026-09-24</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">45 dòng × 14 chỉ số · 2026-07-23 → 2026-09-25</t>
+    <t xml:space="preserve">46 dòng × 14 chỉ số · 2026-07-23 → 2026-09-26</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">45 dòng × 14 chỉ số · 2026-06-30 → 2026-09-25</t>
+    <t xml:space="preserve">46 dòng × 14 chỉ số · 2026-06-30 → 2026-09-26</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">42 dòng × 11 chỉ số · 2026-07-27 → 2026-09-25</t>
+    <t xml:space="preserve">43 dòng × 11 chỉ số · 2026-07-27 → 2026-09-26</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 81 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 82 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 45 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 46 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 45 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 46 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 42 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 43 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -978,7 +978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3156,6 +3156,32 @@
       </c>
       <c r="H86" s="16" t="n">
         <v>45</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="15" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B87" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C87" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>124</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="F87" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H87" s="16" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -3174,7 +3200,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5403,6 +5429,53 @@
       </c>
       <c r="O50" s="16" t="n">
         <v>635</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="15" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B51" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="D51" s="16" t="n">
+        <v>4509</v>
+      </c>
+      <c r="E51" s="16" t="n">
+        <v>433</v>
+      </c>
+      <c r="F51" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G51" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>86</v>
+      </c>
+      <c r="I51" s="16" t="n">
+        <v>2397</v>
+      </c>
+      <c r="J51" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K51" s="16" t="n">
+        <v>1229</v>
+      </c>
+      <c r="L51" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="M51" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="N51" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O51" s="16" t="n">
+        <v>634</v>
       </c>
     </row>
   </sheetData>
@@ -5421,7 +5494,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7554,6 +7627,53 @@
       </c>
       <c r="O50" s="16" t="n">
         <v>336</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="15" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B51" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <v>701</v>
+      </c>
+      <c r="D51" s="16" t="n">
+        <v>665</v>
+      </c>
+      <c r="E51" s="19" t="n">
+        <v>34.59</v>
+      </c>
+      <c r="F51" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" s="16" t="n">
+        <v>558</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>387</v>
+      </c>
+      <c r="I51" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="J51" s="19" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K51" s="16" t="n">
+        <v>1013</v>
+      </c>
+      <c r="L51" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="M51" s="16" t="n">
+        <v>81</v>
+      </c>
+      <c r="N51" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O51" s="16" t="n">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -7572,7 +7692,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9126,6 +9246,44 @@
       </c>
       <c r="L47" s="16" t="n">
         <v>239208</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="15" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B48" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="C48" s="16" t="n">
+        <v>96</v>
+      </c>
+      <c r="D48" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E48" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F48" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G48" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H48" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I48" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="J48" s="16" t="n">
+        <v>337</v>
+      </c>
+      <c r="K48" s="16" t="n">
+        <v>271</v>
+      </c>
+      <c r="L48" s="16" t="n">
+        <v>239577</v>
       </c>
     </row>
   </sheetData>
@@ -9190,16 +9348,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>118</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9207,16 +9365,16 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>345</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>347</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9224,16 +9382,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>3969</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>4093</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9241,16 +9399,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>380</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>396</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9258,15 +9416,15 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>13</v>
       </c>
     </row>
@@ -9275,16 +9433,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>147</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>149</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9292,16 +9450,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H86,'Social — theo ngày'!$A$6:$A$86,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$86,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2157</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2186</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9336,7 +9494,7 @@
         <v>115</v>
       </c>
       <c r="D17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B50</f>
+        <f aca="false">'Social — 28 ngày'!B51</f>
         <v>116</v>
       </c>
     </row>
@@ -9353,8 +9511,8 @@
         <v>184</v>
       </c>
       <c r="D18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C50</f>
-        <v>135</v>
+        <f aca="false">'Social — 28 ngày'!C51</f>
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9370,8 +9528,8 @@
         <v>4735</v>
       </c>
       <c r="D19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D50</f>
-        <v>4560</v>
+        <f aca="false">'Social — 28 ngày'!D51</f>
+        <v>4509</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9387,8 +9545,8 @@
         <v>280</v>
       </c>
       <c r="D20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E50</f>
-        <v>486</v>
+        <f aca="false">'Social — 28 ngày'!E51</f>
+        <v>433</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9404,7 +9562,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F50</f>
+        <f aca="false">'Social — 28 ngày'!F51</f>
         <v>49</v>
       </c>
     </row>
@@ -9421,7 +9579,7 @@
         <v>68</v>
       </c>
       <c r="D22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G50</f>
+        <f aca="false">'Social — 28 ngày'!G51</f>
         <v>15</v>
       </c>
     </row>
@@ -9438,7 +9596,7 @@
         <v>275</v>
       </c>
       <c r="D23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H50</f>
+        <f aca="false">'Social — 28 ngày'!H51</f>
         <v>86</v>
       </c>
     </row>
@@ -9455,8 +9613,8 @@
         <v>1039</v>
       </c>
       <c r="D24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I50</f>
-        <v>2422</v>
+        <f aca="false">'Social — 28 ngày'!I51</f>
+        <v>2397</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9472,7 +9630,7 @@
         <v>100</v>
       </c>
       <c r="D25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J50</f>
+        <f aca="false">'Social — 28 ngày'!J51</f>
         <v>102</v>
       </c>
     </row>
@@ -9489,8 +9647,8 @@
         <v>1691</v>
       </c>
       <c r="D26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K50</f>
-        <v>1328</v>
+        <f aca="false">'Social — 28 ngày'!K51</f>
+        <v>1229</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9506,8 +9664,8 @@
         <v>127</v>
       </c>
       <c r="D27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L50</f>
-        <v>33</v>
+        <f aca="false">'Social — 28 ngày'!L51</f>
+        <v>28</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9523,8 +9681,8 @@
         <v>86</v>
       </c>
       <c r="D28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M50</f>
-        <v>59</v>
+        <f aca="false">'Social — 28 ngày'!M51</f>
+        <v>44</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9540,7 +9698,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N50</f>
+        <f aca="false">'Social — 28 ngày'!N51</f>
         <v>4</v>
       </c>
     </row>
@@ -9557,8 +9715,8 @@
         <v>59</v>
       </c>
       <c r="D30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O50</f>
-        <v>635</v>
+        <f aca="false">'Social — 28 ngày'!O51</f>
+        <v>634</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9600,8 +9758,8 @@
         <v>21</v>
       </c>
       <c r="E34" s="24" t="n">
-        <f aca="false">SEO!B50</f>
-        <v>12</v>
+        <f aca="false">SEO!B51</f>
+        <v>14</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9621,8 +9779,8 @@
         <v>364</v>
       </c>
       <c r="E35" s="24" t="n">
-        <f aca="false">SEO!C50</f>
-        <v>699</v>
+        <f aca="false">SEO!C51</f>
+        <v>701</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9642,8 +9800,8 @@
         <v>349</v>
       </c>
       <c r="E36" s="24" t="n">
-        <f aca="false">SEO!D50</f>
-        <v>663</v>
+        <f aca="false">SEO!D51</f>
+        <v>665</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9663,8 +9821,8 @@
         <v>42.93</v>
       </c>
       <c r="E37" s="24" t="n">
-        <f aca="false">SEO!E50</f>
-        <v>33.9</v>
+        <f aca="false">SEO!E51</f>
+        <v>34.59</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9684,7 +9842,7 @@
         <v>7</v>
       </c>
       <c r="E38" s="24" t="n">
-        <f aca="false">SEO!F50</f>
+        <f aca="false">SEO!F51</f>
         <v>3</v>
       </c>
     </row>
@@ -9705,8 +9863,8 @@
         <v>375</v>
       </c>
       <c r="E39" s="24" t="n">
-        <f aca="false">SEO!G50</f>
-        <v>584</v>
+        <f aca="false">SEO!G51</f>
+        <v>558</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9726,8 +9884,8 @@
         <v>204</v>
       </c>
       <c r="E40" s="24" t="n">
-        <f aca="false">SEO!H50</f>
-        <v>399</v>
+        <f aca="false">SEO!H51</f>
+        <v>387</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9747,7 +9905,7 @@
         <v>67</v>
       </c>
       <c r="E41" s="24" t="n">
-        <f aca="false">SEO!I50</f>
+        <f aca="false">SEO!I51</f>
         <v>34</v>
       </c>
     </row>
@@ -9768,8 +9926,8 @@
         <v>3.8</v>
       </c>
       <c r="E42" s="24" t="n">
-        <f aca="false">SEO!J50</f>
-        <v>3.3</v>
+        <f aca="false">SEO!J51</f>
+        <v>3.4</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9789,8 +9947,8 @@
         <v>1757</v>
       </c>
       <c r="E43" s="24" t="n">
-        <f aca="false">SEO!K50</f>
-        <v>1034</v>
+        <f aca="false">SEO!K51</f>
+        <v>1013</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9810,8 +9968,8 @@
         <v>29.4</v>
       </c>
       <c r="E44" s="24" t="n">
-        <f aca="false">SEO!L50</f>
-        <v>29.1</v>
+        <f aca="false">SEO!L51</f>
+        <v>28</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9831,8 +9989,8 @@
         <v>151</v>
       </c>
       <c r="E45" s="24" t="n">
-        <f aca="false">SEO!M50</f>
-        <v>86</v>
+        <f aca="false">SEO!M51</f>
+        <v>81</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9852,7 +10010,7 @@
         <v>95</v>
       </c>
       <c r="E46" s="24" t="n">
-        <f aca="false">SEO!N50</f>
+        <f aca="false">SEO!N51</f>
         <v>119</v>
       </c>
     </row>
@@ -9873,8 +10031,8 @@
         <v>1022</v>
       </c>
       <c r="E47" s="24" t="n">
-        <f aca="false">SEO!O50</f>
-        <v>336</v>
+        <f aca="false">SEO!O51</f>
+        <v>337</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9909,7 +10067,7 @@
         <v>88</v>
       </c>
       <c r="D51" s="24" t="n">
-        <f aca="false">Audit!B47</f>
+        <f aca="false">Audit!B48</f>
         <v>92</v>
       </c>
     </row>
@@ -9926,8 +10084,8 @@
         <v>97</v>
       </c>
       <c r="D52" s="24" t="n">
-        <f aca="false">Audit!C47</f>
-        <v>93</v>
+        <f aca="false">Audit!C48</f>
+        <v>96</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9943,8 +10101,8 @@
         <v>92</v>
       </c>
       <c r="D53" s="24" t="n">
-        <f aca="false">Audit!D47</f>
-        <v>93</v>
+        <f aca="false">Audit!D48</f>
+        <v>95</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9960,7 +10118,7 @@
         <v>91</v>
       </c>
       <c r="D54" s="24" t="n">
-        <f aca="false">Audit!E47</f>
+        <f aca="false">Audit!E48</f>
         <v>92</v>
       </c>
     </row>
@@ -9977,7 +10135,7 @@
         <v>91</v>
       </c>
       <c r="D55" s="24" t="n">
-        <f aca="false">Audit!F47</f>
+        <f aca="false">Audit!F48</f>
         <v>118</v>
       </c>
     </row>
@@ -9994,7 +10152,7 @@
         <v>88</v>
       </c>
       <c r="D56" s="24" t="n">
-        <f aca="false">Audit!G47</f>
+        <f aca="false">Audit!G48</f>
         <v>98</v>
       </c>
     </row>
@@ -10011,7 +10169,7 @@
         <v>92</v>
       </c>
       <c r="D57" s="24" t="n">
-        <f aca="false">Audit!H47</f>
+        <f aca="false">Audit!H48</f>
         <v>119</v>
       </c>
     </row>
@@ -10028,8 +10186,8 @@
         <v>96</v>
       </c>
       <c r="D58" s="24" t="n">
-        <f aca="false">Audit!I47</f>
-        <v>88</v>
+        <f aca="false">Audit!I48</f>
+        <v>92</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10045,8 +10203,8 @@
         <v>862</v>
       </c>
       <c r="D59" s="24" t="n">
-        <f aca="false">Audit!J47</f>
-        <v>336</v>
+        <f aca="false">Audit!J48</f>
+        <v>337</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10062,8 +10220,8 @@
         <v>0</v>
       </c>
       <c r="D60" s="24" t="n">
-        <f aca="false">Audit!K47</f>
-        <v>274</v>
+        <f aca="false">Audit!K48</f>
+        <v>271</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10079,8 +10237,8 @@
         <v>0</v>
       </c>
       <c r="D61" s="24" t="n">
-        <f aca="false">Audit!L47</f>
-        <v>239208</v>
+        <f aca="false">Audit!L48</f>
+        <v>239577</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel 2026-09-28: rebuild dxl-metrics.xlsx from the three fresh rollups (recalc 152 formulas, 0 errors)
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-09-26 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-09-28 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">82 dòng × 7 chỉ số · 2026-07-05 → 2026-09-24</t>
+    <t xml:space="preserve">84 dòng × 7 chỉ số · 2026-07-05 → 2026-09-26</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">46 dòng × 14 chỉ số · 2026-07-23 → 2026-09-26</t>
+    <t xml:space="preserve">47 dòng × 14 chỉ số · 2026-07-23 → 2026-09-28</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">46 dòng × 14 chỉ số · 2026-06-30 → 2026-09-26</t>
+    <t xml:space="preserve">47 dòng × 14 chỉ số · 2026-06-30 → 2026-09-28</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">43 dòng × 11 chỉ số · 2026-07-27 → 2026-09-26</t>
+    <t xml:space="preserve">44 dòng × 11 chỉ số · 2026-07-27 → 2026-09-28</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 82 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 84 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 46 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 47 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 46 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 47 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 43 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 44 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -978,7 +978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3182,6 +3182,58 @@
       </c>
       <c r="H87" s="16" t="n">
         <v>29</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="15" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B88" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="C88" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="16" t="n">
+        <v>130</v>
+      </c>
+      <c r="E88" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="F88" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G88" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H88" s="16" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="15" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B89" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="16" t="n">
+        <v>51</v>
+      </c>
+      <c r="E89" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="F89" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="16" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3200,7 +3252,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5475,6 +5527,53 @@
         <v>4</v>
       </c>
       <c r="O51" s="16" t="n">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="15" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B52" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <v>144</v>
+      </c>
+      <c r="D52" s="16" t="n">
+        <v>4483</v>
+      </c>
+      <c r="E52" s="16" t="n">
+        <v>445</v>
+      </c>
+      <c r="F52" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G52" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="H52" s="16" t="n">
+        <v>87</v>
+      </c>
+      <c r="I52" s="16" t="n">
+        <v>2320</v>
+      </c>
+      <c r="J52" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K52" s="16" t="n">
+        <v>1232</v>
+      </c>
+      <c r="L52" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="M52" s="16" t="n">
+        <v>43</v>
+      </c>
+      <c r="N52" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O52" s="16" t="n">
         <v>634</v>
       </c>
     </row>
@@ -5494,7 +5593,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7674,6 +7773,53 @@
       </c>
       <c r="O51" s="16" t="n">
         <v>337</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="15" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B52" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <v>745</v>
+      </c>
+      <c r="D52" s="16" t="n">
+        <v>709</v>
+      </c>
+      <c r="E52" s="19" t="n">
+        <v>33.88</v>
+      </c>
+      <c r="F52" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="16" t="n">
+        <v>552</v>
+      </c>
+      <c r="H52" s="16" t="n">
+        <v>392</v>
+      </c>
+      <c r="I52" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="J52" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" s="16" t="n">
+        <v>1039</v>
+      </c>
+      <c r="L52" s="19" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="M52" s="16" t="n">
+        <v>78</v>
+      </c>
+      <c r="N52" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O52" s="16" t="n">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -7692,7 +7838,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9283,6 +9429,44 @@
         <v>271</v>
       </c>
       <c r="L48" s="16" t="n">
+        <v>239577</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="15" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B49" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="C49" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="D49" s="16" t="n">
+        <v>94</v>
+      </c>
+      <c r="E49" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F49" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G49" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H49" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I49" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="J49" s="16" t="n">
+        <v>334</v>
+      </c>
+      <c r="K49" s="16" t="n">
+        <v>268</v>
+      </c>
+      <c r="L49" s="16" t="n">
         <v>239577</v>
       </c>
     </row>
@@ -9348,16 +9532,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>124</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9365,15 +9549,15 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>347</v>
       </c>
     </row>
@@ -9382,16 +9566,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>4093</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>4274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9399,16 +9583,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>396</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>412</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9416,16 +9600,16 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>13</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9433,16 +9617,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>149</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>155</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9450,16 +9634,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H87,'Social — theo ngày'!$A$6:$A$87,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$87,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2186</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2220</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9494,7 +9678,7 @@
         <v>115</v>
       </c>
       <c r="D17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B51</f>
+        <f aca="false">'Social — 28 ngày'!B52</f>
         <v>116</v>
       </c>
     </row>
@@ -9511,8 +9695,8 @@
         <v>184</v>
       </c>
       <c r="D18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C51</f>
-        <v>140</v>
+        <f aca="false">'Social — 28 ngày'!C52</f>
+        <v>144</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9528,8 +9712,8 @@
         <v>4735</v>
       </c>
       <c r="D19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D51</f>
-        <v>4509</v>
+        <f aca="false">'Social — 28 ngày'!D52</f>
+        <v>4483</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9545,8 +9729,8 @@
         <v>280</v>
       </c>
       <c r="D20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E51</f>
-        <v>433</v>
+        <f aca="false">'Social — 28 ngày'!E52</f>
+        <v>445</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9562,7 +9746,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F51</f>
+        <f aca="false">'Social — 28 ngày'!F52</f>
         <v>49</v>
       </c>
     </row>
@@ -9579,8 +9763,8 @@
         <v>68</v>
       </c>
       <c r="D22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G51</f>
-        <v>15</v>
+        <f aca="false">'Social — 28 ngày'!G52</f>
+        <v>18</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9596,8 +9780,8 @@
         <v>275</v>
       </c>
       <c r="D23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H51</f>
-        <v>86</v>
+        <f aca="false">'Social — 28 ngày'!H52</f>
+        <v>87</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9613,8 +9797,8 @@
         <v>1039</v>
       </c>
       <c r="D24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I51</f>
-        <v>2397</v>
+        <f aca="false">'Social — 28 ngày'!I52</f>
+        <v>2320</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9630,7 +9814,7 @@
         <v>100</v>
       </c>
       <c r="D25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J51</f>
+        <f aca="false">'Social — 28 ngày'!J52</f>
         <v>102</v>
       </c>
     </row>
@@ -9647,8 +9831,8 @@
         <v>1691</v>
       </c>
       <c r="D26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K51</f>
-        <v>1229</v>
+        <f aca="false">'Social — 28 ngày'!K52</f>
+        <v>1232</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9664,8 +9848,8 @@
         <v>127</v>
       </c>
       <c r="D27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L51</f>
-        <v>28</v>
+        <f aca="false">'Social — 28 ngày'!L52</f>
+        <v>27</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9681,8 +9865,8 @@
         <v>86</v>
       </c>
       <c r="D28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M51</f>
-        <v>44</v>
+        <f aca="false">'Social — 28 ngày'!M52</f>
+        <v>43</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9698,7 +9882,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N51</f>
+        <f aca="false">'Social — 28 ngày'!N52</f>
         <v>4</v>
       </c>
     </row>
@@ -9715,7 +9899,7 @@
         <v>59</v>
       </c>
       <c r="D30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O51</f>
+        <f aca="false">'Social — 28 ngày'!O52</f>
         <v>634</v>
       </c>
     </row>
@@ -9758,8 +9942,8 @@
         <v>21</v>
       </c>
       <c r="E34" s="24" t="n">
-        <f aca="false">SEO!B51</f>
-        <v>14</v>
+        <f aca="false">SEO!B52</f>
+        <v>17</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9779,8 +9963,8 @@
         <v>364</v>
       </c>
       <c r="E35" s="24" t="n">
-        <f aca="false">SEO!C51</f>
-        <v>701</v>
+        <f aca="false">SEO!C52</f>
+        <v>745</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9800,8 +9984,8 @@
         <v>349</v>
       </c>
       <c r="E36" s="24" t="n">
-        <f aca="false">SEO!D51</f>
-        <v>665</v>
+        <f aca="false">SEO!D52</f>
+        <v>709</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9821,8 +10005,8 @@
         <v>42.93</v>
       </c>
       <c r="E37" s="24" t="n">
-        <f aca="false">SEO!E51</f>
-        <v>34.59</v>
+        <f aca="false">SEO!E52</f>
+        <v>33.88</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9842,7 +10026,7 @@
         <v>7</v>
       </c>
       <c r="E38" s="24" t="n">
-        <f aca="false">SEO!F51</f>
+        <f aca="false">SEO!F52</f>
         <v>3</v>
       </c>
     </row>
@@ -9863,8 +10047,8 @@
         <v>375</v>
       </c>
       <c r="E39" s="24" t="n">
-        <f aca="false">SEO!G51</f>
-        <v>558</v>
+        <f aca="false">SEO!G52</f>
+        <v>552</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9884,8 +10068,8 @@
         <v>204</v>
       </c>
       <c r="E40" s="24" t="n">
-        <f aca="false">SEO!H51</f>
-        <v>387</v>
+        <f aca="false">SEO!H52</f>
+        <v>392</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9905,8 +10089,8 @@
         <v>67</v>
       </c>
       <c r="E41" s="24" t="n">
-        <f aca="false">SEO!I51</f>
-        <v>34</v>
+        <f aca="false">SEO!I52</f>
+        <v>31</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9926,8 +10110,8 @@
         <v>3.8</v>
       </c>
       <c r="E42" s="24" t="n">
-        <f aca="false">SEO!J51</f>
-        <v>3.4</v>
+        <f aca="false">SEO!J52</f>
+        <v>3</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9947,8 +10131,8 @@
         <v>1757</v>
       </c>
       <c r="E43" s="24" t="n">
-        <f aca="false">SEO!K51</f>
-        <v>1013</v>
+        <f aca="false">SEO!K52</f>
+        <v>1039</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9968,8 +10152,8 @@
         <v>29.4</v>
       </c>
       <c r="E44" s="24" t="n">
-        <f aca="false">SEO!L51</f>
-        <v>28</v>
+        <f aca="false">SEO!L52</f>
+        <v>26.6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9989,8 +10173,8 @@
         <v>151</v>
       </c>
       <c r="E45" s="24" t="n">
-        <f aca="false">SEO!M51</f>
-        <v>81</v>
+        <f aca="false">SEO!M52</f>
+        <v>78</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10010,7 +10194,7 @@
         <v>95</v>
       </c>
       <c r="E46" s="24" t="n">
-        <f aca="false">SEO!N51</f>
+        <f aca="false">SEO!N52</f>
         <v>119</v>
       </c>
     </row>
@@ -10031,8 +10215,8 @@
         <v>1022</v>
       </c>
       <c r="E47" s="24" t="n">
-        <f aca="false">SEO!O51</f>
-        <v>337</v>
+        <f aca="false">SEO!O52</f>
+        <v>334</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10067,7 +10251,7 @@
         <v>88</v>
       </c>
       <c r="D51" s="24" t="n">
-        <f aca="false">Audit!B48</f>
+        <f aca="false">Audit!B49</f>
         <v>92</v>
       </c>
     </row>
@@ -10084,8 +10268,8 @@
         <v>97</v>
       </c>
       <c r="D52" s="24" t="n">
-        <f aca="false">Audit!C48</f>
-        <v>96</v>
+        <f aca="false">Audit!C49</f>
+        <v>95</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10101,8 +10285,8 @@
         <v>92</v>
       </c>
       <c r="D53" s="24" t="n">
-        <f aca="false">Audit!D48</f>
-        <v>95</v>
+        <f aca="false">Audit!D49</f>
+        <v>94</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10118,7 +10302,7 @@
         <v>91</v>
       </c>
       <c r="D54" s="24" t="n">
-        <f aca="false">Audit!E48</f>
+        <f aca="false">Audit!E49</f>
         <v>92</v>
       </c>
     </row>
@@ -10135,7 +10319,7 @@
         <v>91</v>
       </c>
       <c r="D55" s="24" t="n">
-        <f aca="false">Audit!F48</f>
+        <f aca="false">Audit!F49</f>
         <v>118</v>
       </c>
     </row>
@@ -10152,7 +10336,7 @@
         <v>88</v>
       </c>
       <c r="D56" s="24" t="n">
-        <f aca="false">Audit!G48</f>
+        <f aca="false">Audit!G49</f>
         <v>98</v>
       </c>
     </row>
@@ -10169,7 +10353,7 @@
         <v>92</v>
       </c>
       <c r="D57" s="24" t="n">
-        <f aca="false">Audit!H48</f>
+        <f aca="false">Audit!H49</f>
         <v>119</v>
       </c>
     </row>
@@ -10186,7 +10370,7 @@
         <v>96</v>
       </c>
       <c r="D58" s="24" t="n">
-        <f aca="false">Audit!I48</f>
+        <f aca="false">Audit!I49</f>
         <v>92</v>
       </c>
     </row>
@@ -10203,8 +10387,8 @@
         <v>862</v>
       </c>
       <c r="D59" s="24" t="n">
-        <f aca="false">Audit!J48</f>
-        <v>337</v>
+        <f aca="false">Audit!J49</f>
+        <v>334</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10220,8 +10404,8 @@
         <v>0</v>
       </c>
       <c r="D60" s="24" t="n">
-        <f aca="false">Audit!K48</f>
-        <v>271</v>
+        <f aca="false">Audit!K49</f>
+        <v>268</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10237,7 +10421,7 @@
         <v>0</v>
       </c>
       <c r="D61" s="24" t="n">
-        <f aca="false">Audit!L48</f>
+        <f aca="false">Audit!L49</f>
         <v>239577</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel 2026-09-29: rebuild dxl-metrics.xlsx from the three fresh rollups (recalc 152 formulas, 0 errors)
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-09-28 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-09-29 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">84 dòng × 7 chỉ số · 2026-07-05 → 2026-09-26</t>
+    <t xml:space="preserve">85 dòng × 7 chỉ số · 2026-07-05 → 2026-09-27</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">47 dòng × 14 chỉ số · 2026-07-23 → 2026-09-28</t>
+    <t xml:space="preserve">48 dòng × 14 chỉ số · 2026-07-23 → 2026-09-29</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">47 dòng × 14 chỉ số · 2026-06-30 → 2026-09-28</t>
+    <t xml:space="preserve">48 dòng × 14 chỉ số · 2026-06-30 → 2026-09-29</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">44 dòng × 11 chỉ số · 2026-07-27 → 2026-09-28</t>
+    <t xml:space="preserve">45 dòng × 11 chỉ số · 2026-07-27 → 2026-09-29</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 84 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 85 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 47 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 48 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 47 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 48 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 44 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 45 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -978,7 +978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3234,6 +3234,32 @@
       </c>
       <c r="H89" s="16" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="15" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B90" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D90" s="16" t="n">
+        <v>65</v>
+      </c>
+      <c r="E90" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F90" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H90" s="16" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -3252,7 +3278,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5574,6 +5600,53 @@
         <v>4</v>
       </c>
       <c r="O52" s="16" t="n">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B53" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C53" s="16" t="n">
+        <v>138</v>
+      </c>
+      <c r="D53" s="16" t="n">
+        <v>4496</v>
+      </c>
+      <c r="E53" s="16" t="n">
+        <v>442</v>
+      </c>
+      <c r="F53" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G53" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="H53" s="16" t="n">
+        <v>87</v>
+      </c>
+      <c r="I53" s="16" t="n">
+        <v>2287</v>
+      </c>
+      <c r="J53" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K53" s="16" t="n">
+        <v>1210</v>
+      </c>
+      <c r="L53" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="M53" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="N53" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O53" s="16" t="n">
         <v>634</v>
       </c>
     </row>
@@ -5593,7 +5666,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7820,6 +7893,53 @@
       </c>
       <c r="O52" s="16" t="n">
         <v>334</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B53" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="C53" s="16" t="n">
+        <v>850</v>
+      </c>
+      <c r="D53" s="16" t="n">
+        <v>814</v>
+      </c>
+      <c r="E53" s="19" t="n">
+        <v>34.59</v>
+      </c>
+      <c r="F53" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G53" s="16" t="n">
+        <v>555</v>
+      </c>
+      <c r="H53" s="16" t="n">
+        <v>393</v>
+      </c>
+      <c r="I53" s="16" t="n">
+        <v>32</v>
+      </c>
+      <c r="J53" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" s="16" t="n">
+        <v>1051</v>
+      </c>
+      <c r="L53" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="M53" s="16" t="n">
+        <v>80</v>
+      </c>
+      <c r="N53" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O53" s="16" t="n">
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -7838,7 +7958,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9468,6 +9588,44 @@
       </c>
       <c r="L49" s="16" t="n">
         <v>239577</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D50" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E50" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G50" s="16" t="n">
+        <v>99</v>
+      </c>
+      <c r="H50" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I50" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="J50" s="16" t="n">
+        <v>323</v>
+      </c>
+      <c r="K50" s="16" t="n">
+        <v>270</v>
+      </c>
+      <c r="L50" s="16" t="n">
+        <v>241329</v>
       </c>
     </row>
   </sheetData>
@@ -9532,15 +9690,15 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>135</v>
       </c>
     </row>
@@ -9549,16 +9707,16 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>347</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>350</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9566,16 +9724,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>4274</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>4339</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9583,16 +9741,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>412</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>416</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9600,15 +9758,15 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>17</v>
       </c>
     </row>
@@ -9617,16 +9775,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>155</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>156</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9634,16 +9792,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H89,'Social — theo ngày'!$A$6:$A$89,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$89,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2220</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2228</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9678,7 +9836,7 @@
         <v>115</v>
       </c>
       <c r="D17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B52</f>
+        <f aca="false">'Social — 28 ngày'!B53</f>
         <v>116</v>
       </c>
     </row>
@@ -9695,8 +9853,8 @@
         <v>184</v>
       </c>
       <c r="D18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C52</f>
-        <v>144</v>
+        <f aca="false">'Social — 28 ngày'!C53</f>
+        <v>138</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9712,8 +9870,8 @@
         <v>4735</v>
       </c>
       <c r="D19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D52</f>
-        <v>4483</v>
+        <f aca="false">'Social — 28 ngày'!D53</f>
+        <v>4496</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9729,8 +9887,8 @@
         <v>280</v>
       </c>
       <c r="D20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E52</f>
-        <v>445</v>
+        <f aca="false">'Social — 28 ngày'!E53</f>
+        <v>442</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9746,7 +9904,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F52</f>
+        <f aca="false">'Social — 28 ngày'!F53</f>
         <v>49</v>
       </c>
     </row>
@@ -9763,8 +9921,8 @@
         <v>68</v>
       </c>
       <c r="D22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G52</f>
-        <v>18</v>
+        <f aca="false">'Social — 28 ngày'!G53</f>
+        <v>17</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9780,7 +9938,7 @@
         <v>275</v>
       </c>
       <c r="D23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H52</f>
+        <f aca="false">'Social — 28 ngày'!H53</f>
         <v>87</v>
       </c>
     </row>
@@ -9797,8 +9955,8 @@
         <v>1039</v>
       </c>
       <c r="D24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I52</f>
-        <v>2320</v>
+        <f aca="false">'Social — 28 ngày'!I53</f>
+        <v>2287</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9814,7 +9972,7 @@
         <v>100</v>
       </c>
       <c r="D25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J52</f>
+        <f aca="false">'Social — 28 ngày'!J53</f>
         <v>102</v>
       </c>
     </row>
@@ -9831,8 +9989,8 @@
         <v>1691</v>
       </c>
       <c r="D26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K52</f>
-        <v>1232</v>
+        <f aca="false">'Social — 28 ngày'!K53</f>
+        <v>1210</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9848,8 +10006,8 @@
         <v>127</v>
       </c>
       <c r="D27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L52</f>
-        <v>27</v>
+        <f aca="false">'Social — 28 ngày'!L53</f>
+        <v>24</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9865,8 +10023,8 @@
         <v>86</v>
       </c>
       <c r="D28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M52</f>
-        <v>43</v>
+        <f aca="false">'Social — 28 ngày'!M53</f>
+        <v>38</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9882,7 +10040,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N52</f>
+        <f aca="false">'Social — 28 ngày'!N53</f>
         <v>4</v>
       </c>
     </row>
@@ -9899,7 +10057,7 @@
         <v>59</v>
       </c>
       <c r="D30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O52</f>
+        <f aca="false">'Social — 28 ngày'!O53</f>
         <v>634</v>
       </c>
     </row>
@@ -9942,7 +10100,7 @@
         <v>21</v>
       </c>
       <c r="E34" s="24" t="n">
-        <f aca="false">SEO!B52</f>
+        <f aca="false">SEO!B53</f>
         <v>17</v>
       </c>
     </row>
@@ -9963,8 +10121,8 @@
         <v>364</v>
       </c>
       <c r="E35" s="24" t="n">
-        <f aca="false">SEO!C52</f>
-        <v>745</v>
+        <f aca="false">SEO!C53</f>
+        <v>850</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9984,8 +10142,8 @@
         <v>349</v>
       </c>
       <c r="E36" s="24" t="n">
-        <f aca="false">SEO!D52</f>
-        <v>709</v>
+        <f aca="false">SEO!D53</f>
+        <v>814</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10005,8 +10163,8 @@
         <v>42.93</v>
       </c>
       <c r="E37" s="24" t="n">
-        <f aca="false">SEO!E52</f>
-        <v>33.88</v>
+        <f aca="false">SEO!E53</f>
+        <v>34.59</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10026,7 +10184,7 @@
         <v>7</v>
       </c>
       <c r="E38" s="24" t="n">
-        <f aca="false">SEO!F52</f>
+        <f aca="false">SEO!F53</f>
         <v>3</v>
       </c>
     </row>
@@ -10047,8 +10205,8 @@
         <v>375</v>
       </c>
       <c r="E39" s="24" t="n">
-        <f aca="false">SEO!G52</f>
-        <v>552</v>
+        <f aca="false">SEO!G53</f>
+        <v>555</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10068,8 +10226,8 @@
         <v>204</v>
       </c>
       <c r="E40" s="24" t="n">
-        <f aca="false">SEO!H52</f>
-        <v>392</v>
+        <f aca="false">SEO!H53</f>
+        <v>393</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10089,8 +10247,8 @@
         <v>67</v>
       </c>
       <c r="E41" s="24" t="n">
-        <f aca="false">SEO!I52</f>
-        <v>31</v>
+        <f aca="false">SEO!I53</f>
+        <v>32</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10110,7 +10268,7 @@
         <v>3.8</v>
       </c>
       <c r="E42" s="24" t="n">
-        <f aca="false">SEO!J52</f>
+        <f aca="false">SEO!J53</f>
         <v>3</v>
       </c>
     </row>
@@ -10131,8 +10289,8 @@
         <v>1757</v>
       </c>
       <c r="E43" s="24" t="n">
-        <f aca="false">SEO!K52</f>
-        <v>1039</v>
+        <f aca="false">SEO!K53</f>
+        <v>1051</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10152,8 +10310,8 @@
         <v>29.4</v>
       </c>
       <c r="E44" s="24" t="n">
-        <f aca="false">SEO!L52</f>
-        <v>26.6</v>
+        <f aca="false">SEO!L53</f>
+        <v>26</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10173,8 +10331,8 @@
         <v>151</v>
       </c>
       <c r="E45" s="24" t="n">
-        <f aca="false">SEO!M52</f>
-        <v>78</v>
+        <f aca="false">SEO!M53</f>
+        <v>80</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10194,7 +10352,7 @@
         <v>95</v>
       </c>
       <c r="E46" s="24" t="n">
-        <f aca="false">SEO!N52</f>
+        <f aca="false">SEO!N53</f>
         <v>119</v>
       </c>
     </row>
@@ -10215,8 +10373,8 @@
         <v>1022</v>
       </c>
       <c r="E47" s="24" t="n">
-        <f aca="false">SEO!O52</f>
-        <v>334</v>
+        <f aca="false">SEO!O53</f>
+        <v>323</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10251,8 +10409,8 @@
         <v>88</v>
       </c>
       <c r="D51" s="24" t="n">
-        <f aca="false">Audit!B49</f>
-        <v>92</v>
+        <f aca="false">Audit!B50</f>
+        <v>93</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10268,8 +10426,8 @@
         <v>97</v>
       </c>
       <c r="D52" s="24" t="n">
-        <f aca="false">Audit!C49</f>
-        <v>95</v>
+        <f aca="false">Audit!C50</f>
+        <v>98</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10285,8 +10443,8 @@
         <v>92</v>
       </c>
       <c r="D53" s="24" t="n">
-        <f aca="false">Audit!D49</f>
-        <v>94</v>
+        <f aca="false">Audit!D50</f>
+        <v>95</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10302,7 +10460,7 @@
         <v>91</v>
       </c>
       <c r="D54" s="24" t="n">
-        <f aca="false">Audit!E49</f>
+        <f aca="false">Audit!E50</f>
         <v>92</v>
       </c>
     </row>
@@ -10319,7 +10477,7 @@
         <v>91</v>
       </c>
       <c r="D55" s="24" t="n">
-        <f aca="false">Audit!F49</f>
+        <f aca="false">Audit!F50</f>
         <v>118</v>
       </c>
     </row>
@@ -10336,8 +10494,8 @@
         <v>88</v>
       </c>
       <c r="D56" s="24" t="n">
-        <f aca="false">Audit!G49</f>
-        <v>98</v>
+        <f aca="false">Audit!G50</f>
+        <v>99</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10353,7 +10511,7 @@
         <v>92</v>
       </c>
       <c r="D57" s="24" t="n">
-        <f aca="false">Audit!H49</f>
+        <f aca="false">Audit!H50</f>
         <v>119</v>
       </c>
     </row>
@@ -10370,7 +10528,7 @@
         <v>96</v>
       </c>
       <c r="D58" s="24" t="n">
-        <f aca="false">Audit!I49</f>
+        <f aca="false">Audit!I50</f>
         <v>92</v>
       </c>
     </row>
@@ -10387,8 +10545,8 @@
         <v>862</v>
       </c>
       <c r="D59" s="24" t="n">
-        <f aca="false">Audit!J49</f>
-        <v>334</v>
+        <f aca="false">Audit!J50</f>
+        <v>323</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10404,8 +10562,8 @@
         <v>0</v>
       </c>
       <c r="D60" s="24" t="n">
-        <f aca="false">Audit!K49</f>
-        <v>268</v>
+        <f aca="false">Audit!K50</f>
+        <v>270</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10421,8 +10579,8 @@
         <v>0</v>
       </c>
       <c r="D61" s="24" t="n">
-        <f aca="false">Audit!L49</f>
-        <v>239577</v>
+        <f aca="false">Audit!L50</f>
+        <v>241329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel 2026-09-30: rebuilt from the three fresh rollups, recalc 0 errors
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-09-29 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-09-30 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">85 dòng × 7 chỉ số · 2026-07-05 → 2026-09-27</t>
+    <t xml:space="preserve">86 dòng × 7 chỉ số · 2026-07-05 → 2026-09-28</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">48 dòng × 14 chỉ số · 2026-07-23 → 2026-09-29</t>
+    <t xml:space="preserve">49 dòng × 14 chỉ số · 2026-07-23 → 2026-09-30</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">48 dòng × 14 chỉ số · 2026-06-30 → 2026-09-29</t>
+    <t xml:space="preserve">49 dòng × 14 chỉ số · 2026-06-30 → 2026-09-30</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">45 dòng × 11 chỉ số · 2026-07-27 → 2026-09-29</t>
+    <t xml:space="preserve">46 dòng × 11 chỉ số · 2026-07-27 → 2026-09-30</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 85 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 86 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 48 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 49 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 48 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 49 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 45 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 46 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -978,7 +978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3260,6 +3260,32 @@
       </c>
       <c r="H90" s="16" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="15" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B91" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C91" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D91" s="16" t="n">
+        <v>180</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F91" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G91" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H91" s="16" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -3278,7 +3304,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5647,6 +5673,53 @@
         <v>4</v>
       </c>
       <c r="O53" s="16" t="n">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B54" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C54" s="16" t="n">
+        <v>141</v>
+      </c>
+      <c r="D54" s="16" t="n">
+        <v>4519</v>
+      </c>
+      <c r="E54" s="16" t="n">
+        <v>422</v>
+      </c>
+      <c r="F54" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G54" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="H54" s="16" t="n">
+        <v>87</v>
+      </c>
+      <c r="I54" s="16" t="n">
+        <v>2258</v>
+      </c>
+      <c r="J54" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K54" s="16" t="n">
+        <v>1193</v>
+      </c>
+      <c r="L54" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="M54" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="N54" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O54" s="16" t="n">
         <v>634</v>
       </c>
     </row>
@@ -5666,7 +5739,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7940,6 +8013,53 @@
       </c>
       <c r="O53" s="16" t="n">
         <v>323</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B54" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C54" s="16" t="n">
+        <v>918</v>
+      </c>
+      <c r="D54" s="16" t="n">
+        <v>882</v>
+      </c>
+      <c r="E54" s="19" t="n">
+        <v>33.99</v>
+      </c>
+      <c r="F54" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" s="16" t="n">
+        <v>559</v>
+      </c>
+      <c r="H54" s="16" t="n">
+        <v>394</v>
+      </c>
+      <c r="I54" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="J54" s="19" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K54" s="16" t="n">
+        <v>1056</v>
+      </c>
+      <c r="L54" s="19" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="M54" s="16" t="n">
+        <v>80</v>
+      </c>
+      <c r="N54" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O54" s="16" t="n">
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -7958,7 +8078,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9625,6 +9745,44 @@
         <v>270</v>
       </c>
       <c r="L50" s="16" t="n">
+        <v>241329</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B51" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D51" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E51" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F51" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G51" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H51" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I51" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="J51" s="16" t="n">
+        <v>342</v>
+      </c>
+      <c r="K51" s="16" t="n">
+        <v>276</v>
+      </c>
+      <c r="L51" s="16" t="n">
         <v>241329</v>
       </c>
     </row>
@@ -9690,16 +9848,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>135</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9707,16 +9865,16 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>350</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>353</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9724,16 +9882,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>4339</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>4519</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9741,16 +9899,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>416</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>422</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9758,16 +9916,16 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>17</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9775,16 +9933,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>156</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>160</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9792,16 +9950,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H90,'Social — theo ngày'!$A$6:$A$90,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$90,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2228</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2258</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9836,7 +9994,7 @@
         <v>115</v>
       </c>
       <c r="D17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B53</f>
+        <f aca="false">'Social — 28 ngày'!B54</f>
         <v>116</v>
       </c>
     </row>
@@ -9853,8 +10011,8 @@
         <v>184</v>
       </c>
       <c r="D18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C53</f>
-        <v>138</v>
+        <f aca="false">'Social — 28 ngày'!C54</f>
+        <v>141</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9870,8 +10028,8 @@
         <v>4735</v>
       </c>
       <c r="D19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D53</f>
-        <v>4496</v>
+        <f aca="false">'Social — 28 ngày'!D54</f>
+        <v>4519</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9887,8 +10045,8 @@
         <v>280</v>
       </c>
       <c r="D20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E53</f>
-        <v>442</v>
+        <f aca="false">'Social — 28 ngày'!E54</f>
+        <v>422</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9904,7 +10062,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F53</f>
+        <f aca="false">'Social — 28 ngày'!F54</f>
         <v>49</v>
       </c>
     </row>
@@ -9921,8 +10079,8 @@
         <v>68</v>
       </c>
       <c r="D22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G53</f>
-        <v>17</v>
+        <f aca="false">'Social — 28 ngày'!G54</f>
+        <v>20</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9938,7 +10096,7 @@
         <v>275</v>
       </c>
       <c r="D23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H53</f>
+        <f aca="false">'Social — 28 ngày'!H54</f>
         <v>87</v>
       </c>
     </row>
@@ -9955,8 +10113,8 @@
         <v>1039</v>
       </c>
       <c r="D24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I53</f>
-        <v>2287</v>
+        <f aca="false">'Social — 28 ngày'!I54</f>
+        <v>2258</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9972,7 +10130,7 @@
         <v>100</v>
       </c>
       <c r="D25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J53</f>
+        <f aca="false">'Social — 28 ngày'!J54</f>
         <v>102</v>
       </c>
     </row>
@@ -9989,8 +10147,8 @@
         <v>1691</v>
       </c>
       <c r="D26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K53</f>
-        <v>1210</v>
+        <f aca="false">'Social — 28 ngày'!K54</f>
+        <v>1193</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10006,7 +10164,7 @@
         <v>127</v>
       </c>
       <c r="D27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L53</f>
+        <f aca="false">'Social — 28 ngày'!L54</f>
         <v>24</v>
       </c>
     </row>
@@ -10023,8 +10181,8 @@
         <v>86</v>
       </c>
       <c r="D28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M53</f>
-        <v>38</v>
+        <f aca="false">'Social — 28 ngày'!M54</f>
+        <v>36</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10040,7 +10198,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N53</f>
+        <f aca="false">'Social — 28 ngày'!N54</f>
         <v>4</v>
       </c>
     </row>
@@ -10057,7 +10215,7 @@
         <v>59</v>
       </c>
       <c r="D30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O53</f>
+        <f aca="false">'Social — 28 ngày'!O54</f>
         <v>634</v>
       </c>
     </row>
@@ -10100,8 +10258,8 @@
         <v>21</v>
       </c>
       <c r="E34" s="24" t="n">
-        <f aca="false">SEO!B53</f>
-        <v>17</v>
+        <f aca="false">SEO!B54</f>
+        <v>16</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10121,8 +10279,8 @@
         <v>364</v>
       </c>
       <c r="E35" s="24" t="n">
-        <f aca="false">SEO!C53</f>
-        <v>850</v>
+        <f aca="false">SEO!C54</f>
+        <v>918</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10142,8 +10300,8 @@
         <v>349</v>
       </c>
       <c r="E36" s="24" t="n">
-        <f aca="false">SEO!D53</f>
-        <v>814</v>
+        <f aca="false">SEO!D54</f>
+        <v>882</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10163,8 +10321,8 @@
         <v>42.93</v>
       </c>
       <c r="E37" s="24" t="n">
-        <f aca="false">SEO!E53</f>
-        <v>34.59</v>
+        <f aca="false">SEO!E54</f>
+        <v>33.99</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10184,8 +10342,8 @@
         <v>7</v>
       </c>
       <c r="E38" s="24" t="n">
-        <f aca="false">SEO!F53</f>
-        <v>3</v>
+        <f aca="false">SEO!F54</f>
+        <v>4</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10205,8 +10363,8 @@
         <v>375</v>
       </c>
       <c r="E39" s="24" t="n">
-        <f aca="false">SEO!G53</f>
-        <v>555</v>
+        <f aca="false">SEO!G54</f>
+        <v>559</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10226,8 +10384,8 @@
         <v>204</v>
       </c>
       <c r="E40" s="24" t="n">
-        <f aca="false">SEO!H53</f>
-        <v>393</v>
+        <f aca="false">SEO!H54</f>
+        <v>394</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10247,8 +10405,8 @@
         <v>67</v>
       </c>
       <c r="E41" s="24" t="n">
-        <f aca="false">SEO!I53</f>
-        <v>32</v>
+        <f aca="false">SEO!I54</f>
+        <v>30</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10268,8 +10426,8 @@
         <v>3.8</v>
       </c>
       <c r="E42" s="24" t="n">
-        <f aca="false">SEO!J53</f>
-        <v>3</v>
+        <f aca="false">SEO!J54</f>
+        <v>2.8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10289,8 +10447,8 @@
         <v>1757</v>
       </c>
       <c r="E43" s="24" t="n">
-        <f aca="false">SEO!K53</f>
-        <v>1051</v>
+        <f aca="false">SEO!K54</f>
+        <v>1056</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10310,8 +10468,8 @@
         <v>29.4</v>
       </c>
       <c r="E44" s="24" t="n">
-        <f aca="false">SEO!L53</f>
-        <v>26</v>
+        <f aca="false">SEO!L54</f>
+        <v>25.8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10331,7 +10489,7 @@
         <v>151</v>
       </c>
       <c r="E45" s="24" t="n">
-        <f aca="false">SEO!M53</f>
+        <f aca="false">SEO!M54</f>
         <v>80</v>
       </c>
     </row>
@@ -10352,7 +10510,7 @@
         <v>95</v>
       </c>
       <c r="E46" s="24" t="n">
-        <f aca="false">SEO!N53</f>
+        <f aca="false">SEO!N54</f>
         <v>119</v>
       </c>
     </row>
@@ -10373,8 +10531,8 @@
         <v>1022</v>
       </c>
       <c r="E47" s="24" t="n">
-        <f aca="false">SEO!O53</f>
-        <v>323</v>
+        <f aca="false">SEO!O54</f>
+        <v>342</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10409,7 +10567,7 @@
         <v>88</v>
       </c>
       <c r="D51" s="24" t="n">
-        <f aca="false">Audit!B50</f>
+        <f aca="false">Audit!B51</f>
         <v>93</v>
       </c>
     </row>
@@ -10426,7 +10584,7 @@
         <v>97</v>
       </c>
       <c r="D52" s="24" t="n">
-        <f aca="false">Audit!C50</f>
+        <f aca="false">Audit!C51</f>
         <v>98</v>
       </c>
     </row>
@@ -10443,7 +10601,7 @@
         <v>92</v>
       </c>
       <c r="D53" s="24" t="n">
-        <f aca="false">Audit!D50</f>
+        <f aca="false">Audit!D51</f>
         <v>95</v>
       </c>
     </row>
@@ -10460,7 +10618,7 @@
         <v>91</v>
       </c>
       <c r="D54" s="24" t="n">
-        <f aca="false">Audit!E50</f>
+        <f aca="false">Audit!E51</f>
         <v>92</v>
       </c>
     </row>
@@ -10477,7 +10635,7 @@
         <v>91</v>
       </c>
       <c r="D55" s="24" t="n">
-        <f aca="false">Audit!F50</f>
+        <f aca="false">Audit!F51</f>
         <v>118</v>
       </c>
     </row>
@@ -10494,8 +10652,8 @@
         <v>88</v>
       </c>
       <c r="D56" s="24" t="n">
-        <f aca="false">Audit!G50</f>
-        <v>99</v>
+        <f aca="false">Audit!G51</f>
+        <v>98</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10511,7 +10669,7 @@
         <v>92</v>
       </c>
       <c r="D57" s="24" t="n">
-        <f aca="false">Audit!H50</f>
+        <f aca="false">Audit!H51</f>
         <v>119</v>
       </c>
     </row>
@@ -10528,7 +10686,7 @@
         <v>96</v>
       </c>
       <c r="D58" s="24" t="n">
-        <f aca="false">Audit!I50</f>
+        <f aca="false">Audit!I51</f>
         <v>92</v>
       </c>
     </row>
@@ -10545,8 +10703,8 @@
         <v>862</v>
       </c>
       <c r="D59" s="24" t="n">
-        <f aca="false">Audit!J50</f>
-        <v>323</v>
+        <f aca="false">Audit!J51</f>
+        <v>342</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10562,8 +10720,8 @@
         <v>0</v>
       </c>
       <c r="D60" s="24" t="n">
-        <f aca="false">Audit!K50</f>
-        <v>270</v>
+        <f aca="false">Audit!K51</f>
+        <v>276</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10579,7 +10737,7 @@
         <v>0</v>
       </c>
       <c r="D61" s="24" t="n">
-        <f aca="false">Audit!L50</f>
+        <f aca="false">Audit!L51</f>
         <v>241329</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social 2026-10-01: window 2-29 Sep, FB views 4,427 up 5.6%, IG 2,297, LI 1,219; YouTube not read (Google sign-out); Excel rebuilt, recalc 0 errors
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="97">
   <si>
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-09-30 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-01 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">86 dòng × 7 chỉ số · 2026-07-05 → 2026-09-28</t>
+    <t xml:space="preserve">87 dòng × 7 chỉ số · 2026-07-05 → 2026-09-29</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">49 dòng × 14 chỉ số · 2026-07-23 → 2026-09-30</t>
+    <t xml:space="preserve">50 dòng × 14 chỉ số · 2026-07-23 → 2026-10-01</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">49 dòng × 14 chỉ số · 2026-06-30 → 2026-09-30</t>
+    <t xml:space="preserve">50 dòng × 14 chỉ số · 2026-06-30 → 2026-10-01</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">46 dòng × 11 chỉ số · 2026-07-27 → 2026-09-30</t>
+    <t xml:space="preserve">47 dòng × 11 chỉ số · 2026-07-27 → 2026-10-01</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 86 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 87 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 49 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 50 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 49 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 50 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 46 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 47 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t xml:space="preserve">KHÔNG CỘNG — Social — 28 ngày (lấy ngày quét cuối tháng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10</t>
   </si>
   <si>
     <t xml:space="preserve">KHÔNG CỘNG — SEO (lấy ngày quét cuối tháng)</t>
@@ -978,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3286,6 +3289,32 @@
       </c>
       <c r="H91" s="16" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B92" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C92" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E92" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G92" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H92" s="16" t="n">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -3304,7 +3333,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5722,6 +5751,49 @@
       <c r="O54" s="16" t="n">
         <v>634</v>
       </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="15" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B55" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C55" s="16" t="n">
+        <v>132</v>
+      </c>
+      <c r="D55" s="16" t="n">
+        <v>4427</v>
+      </c>
+      <c r="E55" s="16" t="n">
+        <v>421</v>
+      </c>
+      <c r="F55" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G55" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="H55" s="16" t="n">
+        <v>87</v>
+      </c>
+      <c r="I55" s="16" t="n">
+        <v>2297</v>
+      </c>
+      <c r="J55" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K55" s="16" t="n">
+        <v>1219</v>
+      </c>
+      <c r="L55" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="M55" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="N55" s="16"/>
+      <c r="O55" s="16"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5739,7 +5811,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8060,6 +8132,35 @@
       </c>
       <c r="O54" s="16" t="n">
         <v>342</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="15" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B55" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="C55" s="16" t="n">
+        <v>918</v>
+      </c>
+      <c r="D55" s="16" t="n">
+        <v>882</v>
+      </c>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
+      <c r="J55" s="16"/>
+      <c r="K55" s="16"/>
+      <c r="L55" s="16"/>
+      <c r="M55" s="16"/>
+      <c r="N55" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O55" s="16" t="n">
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -8078,7 +8179,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9784,6 +9885,44 @@
       </c>
       <c r="L51" s="16" t="n">
         <v>241329</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="15" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B52" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D52" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E52" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F52" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G52" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H52" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I52" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="J52" s="16" t="n">
+        <v>331</v>
+      </c>
+      <c r="K52" s="16" t="n">
+        <v>268</v>
+      </c>
+      <c r="L52" s="16" t="n">
+        <v>241211</v>
       </c>
     </row>
   </sheetData>
@@ -9802,7 +9941,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -9848,16 +9987,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>141</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9865,15 +10004,15 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>353</v>
       </c>
     </row>
@@ -9882,16 +10021,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>4519</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>4614</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9899,15 +10038,15 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>422</v>
       </c>
     </row>
@@ -9916,16 +10055,16 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>20</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>23</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9933,16 +10072,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>160</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>166</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9950,16 +10089,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H91,'Social — theo ngày'!$A$6:$A$91,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$91,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2258</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2318</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9980,6 +10119,9 @@
       <c r="D16" s="21" t="s">
         <v>91</v>
       </c>
+      <c r="E16" s="21" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
@@ -9997,6 +10139,10 @@
         <f aca="false">'Social — 28 ngày'!B54</f>
         <v>116</v>
       </c>
+      <c r="E17" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!B55</f>
+        <v>116</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
@@ -10014,6 +10160,10 @@
         <f aca="false">'Social — 28 ngày'!C54</f>
         <v>141</v>
       </c>
+      <c r="E18" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!C55</f>
+        <v>132</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
@@ -10031,6 +10181,10 @@
         <f aca="false">'Social — 28 ngày'!D54</f>
         <v>4519</v>
       </c>
+      <c r="E19" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!D55</f>
+        <v>4427</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
@@ -10048,6 +10202,10 @@
         <f aca="false">'Social — 28 ngày'!E54</f>
         <v>422</v>
       </c>
+      <c r="E20" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!E55</f>
+        <v>421</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
@@ -10065,6 +10223,10 @@
         <f aca="false">'Social — 28 ngày'!F54</f>
         <v>49</v>
       </c>
+      <c r="E21" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!F55</f>
+        <v>49</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
@@ -10082,6 +10244,10 @@
         <f aca="false">'Social — 28 ngày'!G54</f>
         <v>20</v>
       </c>
+      <c r="E22" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!G55</f>
+        <v>23</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
@@ -10099,6 +10265,10 @@
         <f aca="false">'Social — 28 ngày'!H54</f>
         <v>87</v>
       </c>
+      <c r="E23" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!H55</f>
+        <v>87</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
@@ -10116,6 +10286,10 @@
         <f aca="false">'Social — 28 ngày'!I54</f>
         <v>2258</v>
       </c>
+      <c r="E24" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!I55</f>
+        <v>2297</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
@@ -10133,6 +10307,10 @@
         <f aca="false">'Social — 28 ngày'!J54</f>
         <v>102</v>
       </c>
+      <c r="E25" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!J55</f>
+        <v>102</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="22" t="s">
@@ -10150,6 +10328,10 @@
         <f aca="false">'Social — 28 ngày'!K54</f>
         <v>1193</v>
       </c>
+      <c r="E26" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!K55</f>
+        <v>1219</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
@@ -10167,6 +10349,10 @@
         <f aca="false">'Social — 28 ngày'!L54</f>
         <v>24</v>
       </c>
+      <c r="E27" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!L55</f>
+        <v>26</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="22" t="s">
@@ -10184,6 +10370,10 @@
         <f aca="false">'Social — 28 ngày'!M54</f>
         <v>36</v>
       </c>
+      <c r="E28" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!M55</f>
+        <v>37</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="22" t="s">
@@ -10201,6 +10391,10 @@
         <f aca="false">'Social — 28 ngày'!N54</f>
         <v>4</v>
       </c>
+      <c r="E29" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!N55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
@@ -10218,10 +10412,14 @@
         <f aca="false">'Social — 28 ngày'!O54</f>
         <v>634</v>
       </c>
+      <c r="E30" s="24" t="n">
+        <f aca="false">'Social — 28 ngày'!O55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10229,7 +10427,7 @@
         <v>88</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C33" s="21" t="s">
         <v>89</v>
@@ -10239,6 +10437,9 @@
       </c>
       <c r="E33" s="21" t="s">
         <v>91</v>
+      </c>
+      <c r="F33" s="21" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10261,6 +10462,10 @@
         <f aca="false">SEO!B54</f>
         <v>16</v>
       </c>
+      <c r="F34" s="24" t="n">
+        <f aca="false">SEO!B55</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
@@ -10282,6 +10487,10 @@
         <f aca="false">SEO!C54</f>
         <v>918</v>
       </c>
+      <c r="F35" s="24" t="n">
+        <f aca="false">SEO!C55</f>
+        <v>918</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
@@ -10303,6 +10512,10 @@
         <f aca="false">SEO!D54</f>
         <v>882</v>
       </c>
+      <c r="F36" s="24" t="n">
+        <f aca="false">SEO!D55</f>
+        <v>882</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
@@ -10324,6 +10537,10 @@
         <f aca="false">SEO!E54</f>
         <v>33.99</v>
       </c>
+      <c r="F37" s="24" t="n">
+        <f aca="false">SEO!E55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
@@ -10345,6 +10562,10 @@
         <f aca="false">SEO!F54</f>
         <v>4</v>
       </c>
+      <c r="F38" s="24" t="n">
+        <f aca="false">SEO!F55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
@@ -10366,6 +10587,10 @@
         <f aca="false">SEO!G54</f>
         <v>559</v>
       </c>
+      <c r="F39" s="24" t="n">
+        <f aca="false">SEO!G55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
@@ -10387,6 +10612,10 @@
         <f aca="false">SEO!H54</f>
         <v>394</v>
       </c>
+      <c r="F40" s="24" t="n">
+        <f aca="false">SEO!H55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
@@ -10408,6 +10637,10 @@
         <f aca="false">SEO!I54</f>
         <v>30</v>
       </c>
+      <c r="F41" s="24" t="n">
+        <f aca="false">SEO!I55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
@@ -10429,6 +10662,10 @@
         <f aca="false">SEO!J54</f>
         <v>2.8</v>
       </c>
+      <c r="F42" s="24" t="n">
+        <f aca="false">SEO!J55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22" t="s">
@@ -10450,6 +10687,10 @@
         <f aca="false">SEO!K54</f>
         <v>1056</v>
       </c>
+      <c r="F43" s="24" t="n">
+        <f aca="false">SEO!K55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
@@ -10471,6 +10712,10 @@
         <f aca="false">SEO!L54</f>
         <v>25.8</v>
       </c>
+      <c r="F44" s="24" t="n">
+        <f aca="false">SEO!L55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
@@ -10492,6 +10737,10 @@
         <f aca="false">SEO!M54</f>
         <v>80</v>
       </c>
+      <c r="F45" s="24" t="n">
+        <f aca="false">SEO!M55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="22" t="s">
@@ -10513,6 +10762,10 @@
         <f aca="false">SEO!N54</f>
         <v>119</v>
       </c>
+      <c r="F46" s="24" t="n">
+        <f aca="false">SEO!N55</f>
+        <v>119</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="22" t="s">
@@ -10534,10 +10787,14 @@
         <f aca="false">SEO!O54</f>
         <v>342</v>
       </c>
+      <c r="F47" s="24" t="n">
+        <f aca="false">SEO!O55</f>
+        <v>331</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10553,6 +10810,9 @@
       <c r="D50" s="21" t="s">
         <v>91</v>
       </c>
+      <c r="E50" s="21" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="22" t="s">
@@ -10570,6 +10830,10 @@
         <f aca="false">Audit!B51</f>
         <v>93</v>
       </c>
+      <c r="E51" s="24" t="n">
+        <f aca="false">Audit!B52</f>
+        <v>93</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="22" t="s">
@@ -10587,6 +10851,10 @@
         <f aca="false">Audit!C51</f>
         <v>98</v>
       </c>
+      <c r="E52" s="24" t="n">
+        <f aca="false">Audit!C52</f>
+        <v>98</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="22" t="s">
@@ -10604,6 +10872,10 @@
         <f aca="false">Audit!D51</f>
         <v>95</v>
       </c>
+      <c r="E53" s="24" t="n">
+        <f aca="false">Audit!D52</f>
+        <v>95</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="22" t="s">
@@ -10621,6 +10893,10 @@
         <f aca="false">Audit!E51</f>
         <v>92</v>
       </c>
+      <c r="E54" s="24" t="n">
+        <f aca="false">Audit!E52</f>
+        <v>92</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="22" t="s">
@@ -10638,6 +10914,10 @@
         <f aca="false">Audit!F51</f>
         <v>118</v>
       </c>
+      <c r="E55" s="24" t="n">
+        <f aca="false">Audit!F52</f>
+        <v>118</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="22" t="s">
@@ -10655,6 +10935,10 @@
         <f aca="false">Audit!G51</f>
         <v>98</v>
       </c>
+      <c r="E56" s="24" t="n">
+        <f aca="false">Audit!G52</f>
+        <v>98</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="22" t="s">
@@ -10672,6 +10956,10 @@
         <f aca="false">Audit!H51</f>
         <v>119</v>
       </c>
+      <c r="E57" s="24" t="n">
+        <f aca="false">Audit!H52</f>
+        <v>119</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="22" t="s">
@@ -10689,6 +10977,10 @@
         <f aca="false">Audit!I51</f>
         <v>92</v>
       </c>
+      <c r="E58" s="24" t="n">
+        <f aca="false">Audit!I52</f>
+        <v>92</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="22" t="s">
@@ -10706,6 +10998,10 @@
         <f aca="false">Audit!J51</f>
         <v>342</v>
       </c>
+      <c r="E59" s="24" t="n">
+        <f aca="false">Audit!J52</f>
+        <v>331</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="22" t="s">
@@ -10723,6 +11019,10 @@
         <f aca="false">Audit!K51</f>
         <v>276</v>
       </c>
+      <c r="E60" s="24" t="n">
+        <f aca="false">Audit!K52</f>
+        <v>268</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="22" t="s">
@@ -10739,6 +11039,10 @@
       <c r="D61" s="24" t="n">
         <f aca="false">Audit!L51</f>
         <v>241329</v>
+      </c>
+      <c r="E61" s="24" t="n">
+        <f aca="false">Audit!L52</f>
+        <v>241211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel 2026-10-02: dxl-metrics.xlsx rebuilt from rollups
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-01 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-02 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">87 dòng × 7 chỉ số · 2026-07-05 → 2026-09-29</t>
+    <t xml:space="preserve">88 dòng × 7 chỉ số · 2026-07-05 → 2026-09-30</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">50 dòng × 14 chỉ số · 2026-07-23 → 2026-10-01</t>
+    <t xml:space="preserve">51 dòng × 14 chỉ số · 2026-07-23 → 2026-10-02</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">50 dòng × 14 chỉ số · 2026-06-30 → 2026-10-01</t>
+    <t xml:space="preserve">51 dòng × 14 chỉ số · 2026-06-30 → 2026-10-02</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">47 dòng × 11 chỉ số · 2026-07-27 → 2026-10-01</t>
+    <t xml:space="preserve">48 dòng × 11 chỉ số · 2026-07-27 → 2026-10-02</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 87 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 88 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 50 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 51 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 50 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 51 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 47 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 48 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3315,6 +3315,32 @@
       </c>
       <c r="H92" s="16" t="n">
         <v>60</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B93" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C93" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" s="16" t="n">
+        <v>162</v>
+      </c>
+      <c r="E93" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F93" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G93" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="H93" s="16" t="n">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3333,7 +3359,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5794,6 +5820,53 @@
       </c>
       <c r="N55" s="16"/>
       <c r="O55" s="16"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="15" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B56" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C56" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="D56" s="16" t="n">
+        <v>4339</v>
+      </c>
+      <c r="E56" s="16" t="n">
+        <v>401</v>
+      </c>
+      <c r="F56" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G56" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="H56" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="I56" s="16" t="n">
+        <v>2409</v>
+      </c>
+      <c r="J56" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K56" s="16" t="n">
+        <v>1225</v>
+      </c>
+      <c r="L56" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="M56" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="N56" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="O56" s="16" t="n">
+        <v>633</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5811,7 +5884,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8161,6 +8234,53 @@
       </c>
       <c r="O55" s="16" t="n">
         <v>331</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="15" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B56" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="C56" s="16" t="n">
+        <v>918</v>
+      </c>
+      <c r="D56" s="16" t="n">
+        <v>882</v>
+      </c>
+      <c r="E56" s="19" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="F56" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G56" s="16" t="n">
+        <v>587</v>
+      </c>
+      <c r="H56" s="16" t="n">
+        <v>403</v>
+      </c>
+      <c r="I56" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="J56" s="19" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K56" s="16" t="n">
+        <v>979</v>
+      </c>
+      <c r="L56" s="19" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="M56" s="16" t="n">
+        <v>84</v>
+      </c>
+      <c r="N56" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O56" s="16" t="n">
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -8179,7 +8299,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9922,6 +10042,44 @@
         <v>268</v>
       </c>
       <c r="L52" s="16" t="n">
+        <v>241211</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="15" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B53" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C53" s="16" t="n">
+        <v>99</v>
+      </c>
+      <c r="D53" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E53" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="F53" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G53" s="16" t="n">
+        <v>96</v>
+      </c>
+      <c r="H53" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I53" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="J53" s="16" t="n">
+        <v>531</v>
+      </c>
+      <c r="K53" s="16" t="n">
+        <v>493</v>
+      </c>
+      <c r="L53" s="16" t="n">
         <v>241211</v>
       </c>
     </row>
@@ -9987,16 +10145,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>145</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>160</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10004,16 +10162,16 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>353</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>354</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10021,16 +10179,16 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>4614</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>4776</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10038,16 +10196,16 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>422</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>425</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10055,16 +10213,16 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>23</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10072,16 +10230,16 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>166</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>174</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10089,16 +10247,16 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H92,'Social — theo ngày'!$A$6:$A$92,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$92,"&lt;="&amp;DATE(2026,9,30))</f>
-        <v>2318</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H93,'Social — theo ngày'!$A$6:$A$93,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$93,"&lt;="&amp;DATE(2026,9,30))</f>
+        <v>2465</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10140,7 +10298,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B55</f>
+        <f aca="false">'Social — 28 ngày'!B56</f>
         <v>116</v>
       </c>
     </row>
@@ -10161,8 +10319,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C55</f>
-        <v>132</v>
+        <f aca="false">'Social — 28 ngày'!C56</f>
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10182,8 +10340,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D55</f>
-        <v>4427</v>
+        <f aca="false">'Social — 28 ngày'!D56</f>
+        <v>4339</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10203,8 +10361,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E55</f>
-        <v>421</v>
+        <f aca="false">'Social — 28 ngày'!E56</f>
+        <v>401</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10224,7 +10382,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F55</f>
+        <f aca="false">'Social — 28 ngày'!F56</f>
         <v>49</v>
       </c>
     </row>
@@ -10245,8 +10403,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G55</f>
-        <v>23</v>
+        <f aca="false">'Social — 28 ngày'!G56</f>
+        <v>25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10266,8 +10424,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H55</f>
-        <v>87</v>
+        <f aca="false">'Social — 28 ngày'!H56</f>
+        <v>90</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10287,8 +10445,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I55</f>
-        <v>2297</v>
+        <f aca="false">'Social — 28 ngày'!I56</f>
+        <v>2409</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10308,7 +10466,7 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J55</f>
+        <f aca="false">'Social — 28 ngày'!J56</f>
         <v>102</v>
       </c>
     </row>
@@ -10329,8 +10487,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K55</f>
-        <v>1219</v>
+        <f aca="false">'Social — 28 ngày'!K56</f>
+        <v>1225</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10350,8 +10508,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L55</f>
-        <v>26</v>
+        <f aca="false">'Social — 28 ngày'!L56</f>
+        <v>27</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10371,8 +10529,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M55</f>
-        <v>37</v>
+        <f aca="false">'Social — 28 ngày'!M56</f>
+        <v>35</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10392,8 +10550,8 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N55</f>
-        <v>0</v>
+        <f aca="false">'Social — 28 ngày'!N56</f>
+        <v>6</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10413,8 +10571,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O55</f>
-        <v>0</v>
+        <f aca="false">'Social — 28 ngày'!O56</f>
+        <v>633</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10463,7 +10621,7 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B55</f>
+        <f aca="false">SEO!B56</f>
         <v>18</v>
       </c>
     </row>
@@ -10488,7 +10646,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C55</f>
+        <f aca="false">SEO!C56</f>
         <v>918</v>
       </c>
     </row>
@@ -10513,7 +10671,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D55</f>
+        <f aca="false">SEO!D56</f>
         <v>882</v>
       </c>
     </row>
@@ -10538,8 +10696,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E55</f>
-        <v>0</v>
+        <f aca="false">SEO!E56</f>
+        <v>34.92</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10563,8 +10721,8 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F55</f>
-        <v>0</v>
+        <f aca="false">SEO!F56</f>
+        <v>7</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10588,8 +10746,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G55</f>
-        <v>0</v>
+        <f aca="false">SEO!G56</f>
+        <v>587</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10613,8 +10771,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H55</f>
-        <v>0</v>
+        <f aca="false">SEO!H56</f>
+        <v>403</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10638,8 +10796,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I55</f>
-        <v>0</v>
+        <f aca="false">SEO!I56</f>
+        <v>31</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10663,8 +10821,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J55</f>
-        <v>0</v>
+        <f aca="false">SEO!J56</f>
+        <v>3.2</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10688,8 +10846,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K55</f>
-        <v>0</v>
+        <f aca="false">SEO!K56</f>
+        <v>979</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10713,8 +10871,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L55</f>
-        <v>0</v>
+        <f aca="false">SEO!L56</f>
+        <v>23.6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10738,8 +10896,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M55</f>
-        <v>0</v>
+        <f aca="false">SEO!M56</f>
+        <v>84</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10763,7 +10921,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N55</f>
+        <f aca="false">SEO!N56</f>
         <v>119</v>
       </c>
     </row>
@@ -10788,8 +10946,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O55</f>
-        <v>331</v>
+        <f aca="false">SEO!O56</f>
+        <v>531</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10831,7 +10989,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B52</f>
+        <f aca="false">Audit!B53</f>
         <v>93</v>
       </c>
     </row>
@@ -10852,8 +11010,8 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C52</f>
-        <v>98</v>
+        <f aca="false">Audit!C53</f>
+        <v>99</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10873,7 +11031,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D52</f>
+        <f aca="false">Audit!D53</f>
         <v>95</v>
       </c>
     </row>
@@ -10894,7 +11052,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E52</f>
+        <f aca="false">Audit!E53</f>
         <v>92</v>
       </c>
     </row>
@@ -10915,7 +11073,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F52</f>
+        <f aca="false">Audit!F53</f>
         <v>118</v>
       </c>
     </row>
@@ -10936,8 +11094,8 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G52</f>
-        <v>98</v>
+        <f aca="false">Audit!G53</f>
+        <v>96</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10957,7 +11115,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H52</f>
+        <f aca="false">Audit!H53</f>
         <v>119</v>
       </c>
     </row>
@@ -10978,7 +11136,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I52</f>
+        <f aca="false">Audit!I53</f>
         <v>92</v>
       </c>
     </row>
@@ -10999,8 +11157,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J52</f>
-        <v>331</v>
+        <f aca="false">Audit!J53</f>
+        <v>531</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11020,8 +11178,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K52</f>
-        <v>268</v>
+        <f aca="false">Audit!K53</f>
+        <v>493</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11041,7 +11199,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L52</f>
+        <f aca="false">Audit!L53</f>
         <v>241211</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social: root 2026-10-05 + Excel
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-03 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-04 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">90 dòng × 7 chỉ số · 2026-07-05 → 2026-10-02</t>
+    <t xml:space="preserve">91 dòng × 7 chỉ số · 2026-07-05 → 2026-10-03</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">52 dòng × 14 chỉ số · 2026-07-23 → 2026-10-03</t>
+    <t xml:space="preserve">53 dòng × 14 chỉ số · 2026-07-23 → 2026-10-05</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">52 dòng × 14 chỉ số · 2026-06-30 → 2026-10-03</t>
+    <t xml:space="preserve">53 dòng × 14 chỉ số · 2026-06-30 → 2026-10-05</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">49 dòng × 11 chỉ số · 2026-07-27 → 2026-10-03</t>
+    <t xml:space="preserve">50 dòng × 11 chỉ số · 2026-07-27 → 2026-10-05</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 90 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 91 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 52 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 53 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 52 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 53 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 49 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 50 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -2788,7 +2788,7 @@
         <v>8</v>
       </c>
       <c r="F72" s="16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G72" s="16" t="n">
         <v>14</v>
@@ -2814,7 +2814,7 @@
         <v>12</v>
       </c>
       <c r="F73" s="16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G73" s="16" t="n">
         <v>6</v>
@@ -2918,7 +2918,7 @@
         <v>7</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G77" s="16" t="n">
         <v>3</v>
@@ -2944,7 +2944,7 @@
         <v>77</v>
       </c>
       <c r="F78" s="16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G78" s="16" t="n">
         <v>39</v>
@@ -3393,6 +3393,32 @@
       </c>
       <c r="H95" s="16" t="n">
         <v>183</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="15" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B96" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C96" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D96" s="16" t="n">
+        <v>54</v>
+      </c>
+      <c r="E96" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H96" s="16" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -3411,7 +3437,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -5965,6 +5991,53 @@
       </c>
       <c r="O57" s="16" t="n">
         <v>736</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B58" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <v>158</v>
+      </c>
+      <c r="D58" s="16" t="n">
+        <v>4404</v>
+      </c>
+      <c r="E58" s="16" t="n">
+        <v>401</v>
+      </c>
+      <c r="F58" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G58" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="H58" s="16" t="n">
+        <v>117</v>
+      </c>
+      <c r="I58" s="16" t="n">
+        <v>2616</v>
+      </c>
+      <c r="J58" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K58" s="16" t="n">
+        <v>1282</v>
+      </c>
+      <c r="L58" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="M58" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="N58" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O58" s="16" t="n">
+        <v>938</v>
       </c>
     </row>
   </sheetData>
@@ -5983,7 +6056,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8427,6 +8500,53 @@
       </c>
       <c r="O57" s="19" t="n">
         <v>326.9</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B58" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <v>918</v>
+      </c>
+      <c r="D58" s="16" t="n">
+        <v>882</v>
+      </c>
+      <c r="E58" s="19" t="n">
+        <v>35.18</v>
+      </c>
+      <c r="F58" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G58" s="16" t="n">
+        <v>597</v>
+      </c>
+      <c r="H58" s="16" t="n">
+        <v>414</v>
+      </c>
+      <c r="I58" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="J58" s="19" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K58" s="16" t="n">
+        <v>778</v>
+      </c>
+      <c r="L58" s="19" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="M58" s="16" t="n">
+        <v>83</v>
+      </c>
+      <c r="N58" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O58" s="16" t="n">
+        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -8445,7 +8565,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -10264,6 +10384,44 @@
         <v>274.5</v>
       </c>
       <c r="L54" s="16" t="n">
+        <v>241675</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="15" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B55" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C55" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D55" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E55" s="16" t="n">
+        <v>94</v>
+      </c>
+      <c r="F55" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G55" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H55" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I55" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J55" s="16" t="n">
+        <v>326</v>
+      </c>
+      <c r="K55" s="19" t="n">
+        <v>271.5</v>
+      </c>
+      <c r="L55" s="16" t="n">
         <v>241675</v>
       </c>
     </row>
@@ -10332,20 +10490,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>21</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10353,20 +10511,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>90</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10374,20 +10532,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>383</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>437</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10395,19 +10553,19 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>6</v>
       </c>
     </row>
@@ -10416,20 +10574,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>10</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10437,20 +10595,20 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>174</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>42</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10458,20 +10616,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H95,'Social — theo ngày'!$A$6:$A$95,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$95,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>288</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>305</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10513,7 +10671,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B57</f>
+        <f aca="false">'Social — 28 ngày'!B58</f>
         <v>116</v>
       </c>
     </row>
@@ -10534,8 +10692,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C57</f>
-        <v>157</v>
+        <f aca="false">'Social — 28 ngày'!C58</f>
+        <v>158</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10555,8 +10713,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D57</f>
-        <v>4412</v>
+        <f aca="false">'Social — 28 ngày'!D58</f>
+        <v>4404</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10576,7 +10734,7 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E57</f>
+        <f aca="false">'Social — 28 ngày'!E58</f>
         <v>401</v>
       </c>
     </row>
@@ -10597,7 +10755,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F57</f>
+        <f aca="false">'Social — 28 ngày'!F58</f>
         <v>49</v>
       </c>
     </row>
@@ -10618,8 +10776,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G57</f>
-        <v>32</v>
+        <f aca="false">'Social — 28 ngày'!G58</f>
+        <v>33</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10639,8 +10797,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H57</f>
-        <v>116</v>
+        <f aca="false">'Social — 28 ngày'!H58</f>
+        <v>117</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10660,8 +10818,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I57</f>
-        <v>2610</v>
+        <f aca="false">'Social — 28 ngày'!I58</f>
+        <v>2616</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10681,7 +10839,7 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J57</f>
+        <f aca="false">'Social — 28 ngày'!J58</f>
         <v>102</v>
       </c>
     </row>
@@ -10702,8 +10860,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K57</f>
-        <v>1263</v>
+        <f aca="false">'Social — 28 ngày'!K58</f>
+        <v>1282</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10723,7 +10881,7 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L57</f>
+        <f aca="false">'Social — 28 ngày'!L58</f>
         <v>33</v>
       </c>
     </row>
@@ -10744,8 +10902,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M57</f>
-        <v>34</v>
+        <f aca="false">'Social — 28 ngày'!M58</f>
+        <v>36</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10765,7 +10923,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N57</f>
+        <f aca="false">'Social — 28 ngày'!N58</f>
         <v>7</v>
       </c>
     </row>
@@ -10786,8 +10944,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O57</f>
-        <v>736</v>
+        <f aca="false">'Social — 28 ngày'!O58</f>
+        <v>938</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10836,8 +10994,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B57</f>
-        <v>16</v>
+        <f aca="false">SEO!B58</f>
+        <v>14</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10861,7 +11019,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C57</f>
+        <f aca="false">SEO!C58</f>
         <v>918</v>
       </c>
     </row>
@@ -10886,7 +11044,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D57</f>
+        <f aca="false">SEO!D58</f>
         <v>882</v>
       </c>
     </row>
@@ -10911,8 +11069,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E57</f>
-        <v>35.45</v>
+        <f aca="false">SEO!E58</f>
+        <v>35.18</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10936,7 +11094,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F57</f>
+        <f aca="false">SEO!F58</f>
         <v>7</v>
       </c>
     </row>
@@ -10961,8 +11119,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G57</f>
-        <v>584</v>
+        <f aca="false">SEO!G58</f>
+        <v>597</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10986,8 +11144,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H57</f>
-        <v>402</v>
+        <f aca="false">SEO!H58</f>
+        <v>414</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11011,8 +11169,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I57</f>
-        <v>28</v>
+        <f aca="false">SEO!I58</f>
+        <v>22</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11036,8 +11194,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J57</f>
-        <v>3</v>
+        <f aca="false">SEO!J58</f>
+        <v>2.8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11061,8 +11219,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K57</f>
-        <v>923</v>
+        <f aca="false">SEO!K58</f>
+        <v>778</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11086,8 +11244,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L57</f>
-        <v>22.6</v>
+        <f aca="false">SEO!L58</f>
+        <v>19.3</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11111,8 +11269,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M57</f>
-        <v>86</v>
+        <f aca="false">SEO!M58</f>
+        <v>83</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11136,7 +11294,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N57</f>
+        <f aca="false">SEO!N58</f>
         <v>119</v>
       </c>
     </row>
@@ -11161,8 +11319,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O57</f>
-        <v>326.9</v>
+        <f aca="false">SEO!O58</f>
+        <v>326</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11204,7 +11362,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B54</f>
+        <f aca="false">Audit!B55</f>
         <v>93</v>
       </c>
     </row>
@@ -11225,7 +11383,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C54</f>
+        <f aca="false">Audit!C55</f>
         <v>98</v>
       </c>
     </row>
@@ -11246,7 +11404,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D54</f>
+        <f aca="false">Audit!D55</f>
         <v>97</v>
       </c>
     </row>
@@ -11267,7 +11425,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E54</f>
+        <f aca="false">Audit!E55</f>
         <v>94</v>
       </c>
     </row>
@@ -11288,7 +11446,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F54</f>
+        <f aca="false">Audit!F55</f>
         <v>118</v>
       </c>
     </row>
@@ -11309,7 +11467,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G54</f>
+        <f aca="false">Audit!G55</f>
         <v>98</v>
       </c>
     </row>
@@ -11330,7 +11488,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H54</f>
+        <f aca="false">Audit!H55</f>
         <v>119</v>
       </c>
     </row>
@@ -11351,7 +11509,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I54</f>
+        <f aca="false">Audit!I55</f>
         <v>98</v>
       </c>
     </row>
@@ -11372,8 +11530,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J54</f>
-        <v>327</v>
+        <f aca="false">Audit!J55</f>
+        <v>326</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,8 +11551,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K54</f>
-        <v>274.5</v>
+        <f aca="false">Audit!K55</f>
+        <v>271.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11414,7 +11572,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L54</f>
+        <f aca="false">Audit!L55</f>
         <v>241675</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Hub: Excel 2026-10-06 + weekly report 2026-10-02
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-04 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-05 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">91 dòng × 7 chỉ số · 2026-07-05 → 2026-10-03</t>
+    <t xml:space="preserve">92 dòng × 7 chỉ số · 2026-07-05 → 2026-10-04</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">53 dòng × 14 chỉ số · 2026-07-23 → 2026-10-05</t>
+    <t xml:space="preserve">54 dòng × 14 chỉ số · 2026-07-23 → 2026-10-06</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">53 dòng × 14 chỉ số · 2026-06-30 → 2026-10-05</t>
+    <t xml:space="preserve">54 dòng × 14 chỉ số · 2026-06-30 → 2026-10-06</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">50 dòng × 11 chỉ số · 2026-07-27 → 2026-10-05</t>
+    <t xml:space="preserve">51 dòng × 11 chỉ số · 2026-07-27 → 2026-10-06</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 91 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 92 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 53 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 54 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 53 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 54 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 50 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 51 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3419,6 +3419,32 @@
       </c>
       <c r="H96" s="16" t="n">
         <v>17</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="15" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B97" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D97" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="E97" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" s="16" t="n">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -3437,7 +3463,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6038,6 +6064,53 @@
       </c>
       <c r="O58" s="16" t="n">
         <v>938</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="15" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B59" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C59" s="16" t="n">
+        <v>158</v>
+      </c>
+      <c r="D59" s="16" t="n">
+        <v>4380</v>
+      </c>
+      <c r="E59" s="16" t="n">
+        <v>366</v>
+      </c>
+      <c r="F59" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G59" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="H59" s="16" t="n">
+        <v>117</v>
+      </c>
+      <c r="I59" s="16" t="n">
+        <v>2610</v>
+      </c>
+      <c r="J59" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="K59" s="16" t="n">
+        <v>1253</v>
+      </c>
+      <c r="L59" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="M59" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="N59" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O59" s="16" t="n">
+        <v>940</v>
       </c>
     </row>
   </sheetData>
@@ -6056,7 +6129,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8547,6 +8620,53 @@
       </c>
       <c r="O58" s="16" t="n">
         <v>326</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="15" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B59" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="C59" s="16" t="n">
+        <v>918</v>
+      </c>
+      <c r="D59" s="16" t="n">
+        <v>882</v>
+      </c>
+      <c r="E59" s="19" t="n">
+        <v>34.22</v>
+      </c>
+      <c r="F59" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G59" s="16" t="n">
+        <v>599</v>
+      </c>
+      <c r="H59" s="16" t="n">
+        <v>417</v>
+      </c>
+      <c r="I59" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="J59" s="19" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="K59" s="16" t="n">
+        <v>763</v>
+      </c>
+      <c r="L59" s="19" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="M59" s="16" t="n">
+        <v>83</v>
+      </c>
+      <c r="N59" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O59" s="16" t="n">
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -8565,7 +8685,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -10422,6 +10542,44 @@
         <v>271.5</v>
       </c>
       <c r="L55" s="16" t="n">
+        <v>241675</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="15" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B56" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C56" s="16" t="n">
+        <v>99</v>
+      </c>
+      <c r="D56" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E56" s="16" t="n">
+        <v>94</v>
+      </c>
+      <c r="F56" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G56" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H56" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I56" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J56" s="16" t="n">
+        <v>333</v>
+      </c>
+      <c r="K56" s="19" t="n">
+        <v>282.5</v>
+      </c>
+      <c r="L56" s="16" t="n">
         <v>241675</v>
       </c>
     </row>
@@ -10490,19 +10648,19 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>23</v>
       </c>
     </row>
@@ -10511,20 +10669,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>96</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10532,20 +10690,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>437</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>482</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10553,20 +10711,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>6</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10574,19 +10732,19 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>11</v>
       </c>
     </row>
@@ -10595,20 +10753,20 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>174</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>45</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>46</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10616,20 +10774,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H96,'Social — theo ngày'!$A$6:$A$96,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$96,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>305</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H97,'Social — theo ngày'!$A$6:$A$97,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$97,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>324</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10671,7 +10829,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B58</f>
+        <f aca="false">'Social — 28 ngày'!B59</f>
         <v>116</v>
       </c>
     </row>
@@ -10692,7 +10850,7 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C58</f>
+        <f aca="false">'Social — 28 ngày'!C59</f>
         <v>158</v>
       </c>
     </row>
@@ -10713,8 +10871,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D58</f>
-        <v>4404</v>
+        <f aca="false">'Social — 28 ngày'!D59</f>
+        <v>4380</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10734,8 +10892,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E58</f>
-        <v>401</v>
+        <f aca="false">'Social — 28 ngày'!E59</f>
+        <v>366</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10755,7 +10913,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F58</f>
+        <f aca="false">'Social — 28 ngày'!F59</f>
         <v>49</v>
       </c>
     </row>
@@ -10776,7 +10934,7 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G58</f>
+        <f aca="false">'Social — 28 ngày'!G59</f>
         <v>33</v>
       </c>
     </row>
@@ -10797,7 +10955,7 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H58</f>
+        <f aca="false">'Social — 28 ngày'!H59</f>
         <v>117</v>
       </c>
     </row>
@@ -10818,8 +10976,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I58</f>
-        <v>2616</v>
+        <f aca="false">'Social — 28 ngày'!I59</f>
+        <v>2610</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10839,7 +10997,7 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J58</f>
+        <f aca="false">'Social — 28 ngày'!J59</f>
         <v>102</v>
       </c>
     </row>
@@ -10860,8 +11018,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K58</f>
-        <v>1282</v>
+        <f aca="false">'Social — 28 ngày'!K59</f>
+        <v>1253</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10881,8 +11039,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L58</f>
-        <v>33</v>
+        <f aca="false">'Social — 28 ngày'!L59</f>
+        <v>31</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10902,8 +11060,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M58</f>
-        <v>36</v>
+        <f aca="false">'Social — 28 ngày'!M59</f>
+        <v>37</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10923,7 +11081,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N58</f>
+        <f aca="false">'Social — 28 ngày'!N59</f>
         <v>7</v>
       </c>
     </row>
@@ -10944,8 +11102,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O58</f>
-        <v>938</v>
+        <f aca="false">'Social — 28 ngày'!O59</f>
+        <v>940</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10994,8 +11152,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B58</f>
-        <v>14</v>
+        <f aca="false">SEO!B59</f>
+        <v>13</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11019,7 +11177,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C58</f>
+        <f aca="false">SEO!C59</f>
         <v>918</v>
       </c>
     </row>
@@ -11044,7 +11202,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D58</f>
+        <f aca="false">SEO!D59</f>
         <v>882</v>
       </c>
     </row>
@@ -11069,8 +11227,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E58</f>
-        <v>35.18</v>
+        <f aca="false">SEO!E59</f>
+        <v>34.22</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11094,7 +11252,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F58</f>
+        <f aca="false">SEO!F59</f>
         <v>7</v>
       </c>
     </row>
@@ -11119,8 +11277,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G58</f>
-        <v>597</v>
+        <f aca="false">SEO!G59</f>
+        <v>599</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11144,8 +11302,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H58</f>
-        <v>414</v>
+        <f aca="false">SEO!H59</f>
+        <v>417</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11169,7 +11327,7 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I58</f>
+        <f aca="false">SEO!I59</f>
         <v>22</v>
       </c>
     </row>
@@ -11194,8 +11352,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J58</f>
-        <v>2.8</v>
+        <f aca="false">SEO!J59</f>
+        <v>2.9</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11219,8 +11377,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K58</f>
-        <v>778</v>
+        <f aca="false">SEO!K59</f>
+        <v>763</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11244,8 +11402,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L58</f>
-        <v>19.3</v>
+        <f aca="false">SEO!L59</f>
+        <v>19.6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11269,7 +11427,7 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M58</f>
+        <f aca="false">SEO!M59</f>
         <v>83</v>
       </c>
     </row>
@@ -11294,7 +11452,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N58</f>
+        <f aca="false">SEO!N59</f>
         <v>119</v>
       </c>
     </row>
@@ -11319,8 +11477,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O58</f>
-        <v>326</v>
+        <f aca="false">SEO!O59</f>
+        <v>333</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11362,7 +11520,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B55</f>
+        <f aca="false">Audit!B56</f>
         <v>93</v>
       </c>
     </row>
@@ -11383,8 +11541,8 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C55</f>
-        <v>98</v>
+        <f aca="false">Audit!C56</f>
+        <v>99</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11404,7 +11562,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D55</f>
+        <f aca="false">Audit!D56</f>
         <v>97</v>
       </c>
     </row>
@@ -11425,7 +11583,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E55</f>
+        <f aca="false">Audit!E56</f>
         <v>94</v>
       </c>
     </row>
@@ -11446,7 +11604,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F55</f>
+        <f aca="false">Audit!F56</f>
         <v>118</v>
       </c>
     </row>
@@ -11467,7 +11625,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G55</f>
+        <f aca="false">Audit!G56</f>
         <v>98</v>
       </c>
     </row>
@@ -11488,7 +11646,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H55</f>
+        <f aca="false">Audit!H56</f>
         <v>119</v>
       </c>
     </row>
@@ -11509,7 +11667,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I55</f>
+        <f aca="false">Audit!I56</f>
         <v>98</v>
       </c>
     </row>
@@ -11530,8 +11688,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J55</f>
-        <v>326</v>
+        <f aca="false">Audit!J56</f>
+        <v>333</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11551,8 +11709,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K55</f>
-        <v>271.5</v>
+        <f aca="false">Audit!K56</f>
+        <v>282.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11572,7 +11730,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L55</f>
+        <f aca="false">Audit!L56</f>
         <v>241675</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social: root 2026-10-08 + dxl-metrics.xlsx
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-06 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-07 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">93 dòng × 7 chỉ số · 2026-07-05 → 2026-10-05</t>
+    <t xml:space="preserve">94 dòng × 7 chỉ số · 2026-07-05 → 2026-10-06</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">55 dòng × 14 chỉ số · 2026-07-23 → 2026-10-07</t>
+    <t xml:space="preserve">56 dòng × 14 chỉ số · 2026-07-23 → 2026-10-08</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">55 dòng × 14 chỉ số · 2026-06-30 → 2026-10-07</t>
+    <t xml:space="preserve">56 dòng × 14 chỉ số · 2026-06-30 → 2026-10-08</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">52 dòng × 11 chỉ số · 2026-07-27 → 2026-10-07</t>
+    <t xml:space="preserve">53 dòng × 11 chỉ số · 2026-07-27 → 2026-10-08</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 93 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 94 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 55 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 56 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 55 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 56 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 52 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 53 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3471,6 +3471,32 @@
       </c>
       <c r="H98" s="16" t="n">
         <v>143</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="15" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B99" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="D99" s="16" t="n">
+        <v>521</v>
+      </c>
+      <c r="E99" s="16" t="n">
+        <v>71</v>
+      </c>
+      <c r="F99" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G99" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H99" s="16" t="n">
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3489,7 +3515,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6184,6 +6210,53 @@
       </c>
       <c r="O60" s="16" t="n">
         <v>939</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="15" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B61" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C61" s="16" t="n">
+        <v>198</v>
+      </c>
+      <c r="D61" s="16" t="n">
+        <v>4680</v>
+      </c>
+      <c r="E61" s="16" t="n">
+        <v>393</v>
+      </c>
+      <c r="F61" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G61" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="H61" s="16" t="n">
+        <v>114</v>
+      </c>
+      <c r="I61" s="16" t="n">
+        <v>2794</v>
+      </c>
+      <c r="J61" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="K61" s="16" t="n">
+        <v>1220</v>
+      </c>
+      <c r="L61" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="M61" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="N61" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O61" s="16" t="n">
+        <v>681</v>
       </c>
     </row>
   </sheetData>
@@ -6202,7 +6275,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -8787,6 +8860,53 @@
       </c>
       <c r="O60" s="16" t="n">
         <v>338</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="15" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B61" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C61" s="16" t="n">
+        <v>917</v>
+      </c>
+      <c r="D61" s="16" t="n">
+        <v>881</v>
+      </c>
+      <c r="E61" s="19" t="n">
+        <v>31.01</v>
+      </c>
+      <c r="F61" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G61" s="16" t="n">
+        <v>616</v>
+      </c>
+      <c r="H61" s="16" t="n">
+        <v>432</v>
+      </c>
+      <c r="I61" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="J61" s="19" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="K61" s="16" t="n">
+        <v>748</v>
+      </c>
+      <c r="L61" s="19" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="M61" s="16" t="n">
+        <v>82</v>
+      </c>
+      <c r="N61" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O61" s="16" t="n">
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -8805,7 +8925,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -10738,6 +10858,44 @@
         <v>277.5</v>
       </c>
       <c r="L57" s="16" t="n">
+        <v>241675</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="15" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B58" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <v>99</v>
+      </c>
+      <c r="D58" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E58" s="16" t="n">
+        <v>94</v>
+      </c>
+      <c r="F58" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G58" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H58" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I58" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J58" s="16" t="n">
+        <v>308</v>
+      </c>
+      <c r="K58" s="19" t="n">
+        <v>264.5</v>
+      </c>
+      <c r="L58" s="16" t="n">
         <v>241675</v>
       </c>
     </row>
@@ -10806,20 +10964,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>74</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>78</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10827,20 +10985,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>108</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10848,20 +11006,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>679</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10869,20 +11027,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>21</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>92</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10890,20 +11048,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>11</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10911,20 +11069,20 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>48</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>51</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10932,20 +11090,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H98,'Social — theo ngày'!$A$6:$A$98,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$98,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>467</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H99,'Social — theo ngày'!$A$6:$A$99,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$99,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>638</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10987,7 +11145,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B60</f>
+        <f aca="false">'Social — 28 ngày'!B61</f>
         <v>116</v>
       </c>
     </row>
@@ -11008,8 +11166,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C60</f>
-        <v>201</v>
+        <f aca="false">'Social — 28 ngày'!C61</f>
+        <v>198</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11029,8 +11187,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D60</f>
-        <v>4418</v>
+        <f aca="false">'Social — 28 ngày'!D61</f>
+        <v>4680</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11050,8 +11208,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E60</f>
-        <v>352</v>
+        <f aca="false">'Social — 28 ngày'!E61</f>
+        <v>393</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11071,7 +11229,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F60</f>
+        <f aca="false">'Social — 28 ngày'!F61</f>
         <v>49</v>
       </c>
     </row>
@@ -11092,8 +11250,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G60</f>
-        <v>33</v>
+        <f aca="false">'Social — 28 ngày'!G61</f>
+        <v>35</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11113,8 +11271,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H60</f>
-        <v>119</v>
+        <f aca="false">'Social — 28 ngày'!H61</f>
+        <v>114</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11134,8 +11292,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I60</f>
-        <v>2707</v>
+        <f aca="false">'Social — 28 ngày'!I61</f>
+        <v>2794</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11155,8 +11313,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J60</f>
-        <v>102</v>
+        <f aca="false">'Social — 28 ngày'!J61</f>
+        <v>120</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11176,8 +11334,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K60</f>
-        <v>1188</v>
+        <f aca="false">'Social — 28 ngày'!K61</f>
+        <v>1220</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11197,7 +11355,7 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L60</f>
+        <f aca="false">'Social — 28 ngày'!L61</f>
         <v>29</v>
       </c>
     </row>
@@ -11218,7 +11376,7 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M60</f>
+        <f aca="false">'Social — 28 ngày'!M61</f>
         <v>29</v>
       </c>
     </row>
@@ -11239,7 +11397,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N60</f>
+        <f aca="false">'Social — 28 ngày'!N61</f>
         <v>7</v>
       </c>
     </row>
@@ -11260,8 +11418,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O60</f>
-        <v>939</v>
+        <f aca="false">'Social — 28 ngày'!O61</f>
+        <v>681</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11310,8 +11468,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B60</f>
-        <v>13</v>
+        <f aca="false">SEO!B61</f>
+        <v>12</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11335,8 +11493,8 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C60</f>
-        <v>918</v>
+        <f aca="false">SEO!C61</f>
+        <v>917</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11360,8 +11518,8 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D60</f>
-        <v>882</v>
+        <f aca="false">SEO!D61</f>
+        <v>881</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11385,8 +11543,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E60</f>
-        <v>32.17</v>
+        <f aca="false">SEO!E61</f>
+        <v>31.01</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11410,7 +11568,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F60</f>
+        <f aca="false">SEO!F61</f>
         <v>7</v>
       </c>
     </row>
@@ -11435,8 +11593,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G60</f>
-        <v>600</v>
+        <f aca="false">SEO!G61</f>
+        <v>616</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11460,8 +11618,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H60</f>
-        <v>421</v>
+        <f aca="false">SEO!H61</f>
+        <v>432</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11485,7 +11643,7 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I60</f>
+        <f aca="false">SEO!I61</f>
         <v>22</v>
       </c>
     </row>
@@ -11510,7 +11668,7 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J60</f>
+        <f aca="false">SEO!J61</f>
         <v>2.9</v>
       </c>
     </row>
@@ -11535,7 +11693,7 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K60</f>
+        <f aca="false">SEO!K61</f>
         <v>748</v>
       </c>
     </row>
@@ -11560,7 +11718,7 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L60</f>
+        <f aca="false">SEO!L61</f>
         <v>19.1</v>
       </c>
     </row>
@@ -11585,7 +11743,7 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M60</f>
+        <f aca="false">SEO!M61</f>
         <v>82</v>
       </c>
     </row>
@@ -11610,7 +11768,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N60</f>
+        <f aca="false">SEO!N61</f>
         <v>119</v>
       </c>
     </row>
@@ -11635,8 +11793,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O60</f>
-        <v>338</v>
+        <f aca="false">SEO!O61</f>
+        <v>308</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11678,7 +11836,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B57</f>
+        <f aca="false">Audit!B58</f>
         <v>93</v>
       </c>
     </row>
@@ -11699,8 +11857,8 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C57</f>
-        <v>98</v>
+        <f aca="false">Audit!C58</f>
+        <v>99</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11720,7 +11878,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D57</f>
+        <f aca="false">Audit!D58</f>
         <v>97</v>
       </c>
     </row>
@@ -11741,7 +11899,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E57</f>
+        <f aca="false">Audit!E58</f>
         <v>94</v>
       </c>
     </row>
@@ -11762,7 +11920,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F57</f>
+        <f aca="false">Audit!F58</f>
         <v>118</v>
       </c>
     </row>
@@ -11783,7 +11941,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G57</f>
+        <f aca="false">Audit!G58</f>
         <v>98</v>
       </c>
     </row>
@@ -11804,7 +11962,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H57</f>
+        <f aca="false">Audit!H58</f>
         <v>119</v>
       </c>
     </row>
@@ -11825,7 +11983,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I57</f>
+        <f aca="false">Audit!I58</f>
         <v>98</v>
       </c>
     </row>
@@ -11846,8 +12004,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J57</f>
-        <v>338</v>
+        <f aca="false">Audit!J58</f>
+        <v>308</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11867,8 +12025,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K57</f>
-        <v>277.5</v>
+        <f aca="false">Audit!K58</f>
+        <v>264.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11888,7 +12046,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L57</f>
+        <f aca="false">Audit!L58</f>
         <v>241675</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social: index 2026-10-12 and metrics xlsx
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-08 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-11 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">95 dòng × 7 chỉ số · 2026-07-05 → 2026-10-07</t>
+    <t xml:space="preserve">98 dòng × 7 chỉ số · 2026-07-05 → 2026-10-10</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">57 dòng × 14 chỉ số · 2026-07-23 → 2026-10-09</t>
+    <t xml:space="preserve">58 dòng × 14 chỉ số · 2026-07-23 → 2026-10-12</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">57 dòng × 14 chỉ số · 2026-06-30 → 2026-10-09</t>
+    <t xml:space="preserve">58 dòng × 14 chỉ số · 2026-06-30 → 2026-10-12</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">54 dòng × 11 chỉ số · 2026-07-27 → 2026-10-09</t>
+    <t xml:space="preserve">55 dòng × 11 chỉ số · 2026-07-27 → 2026-10-12</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 95 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 98 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 57 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 58 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 57 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 58 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 54 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 55 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3523,6 +3523,84 @@
       </c>
       <c r="H100" s="16" t="n">
         <v>112</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="15" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B101" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C101" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="D101" s="16" t="n">
+        <v>216</v>
+      </c>
+      <c r="E101" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F101" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G101" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H101" s="16" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="15" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B102" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C102" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="E102" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F102" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H102" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="15" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B103" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="E103" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="16" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -3541,7 +3619,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6330,6 +6408,53 @@
       </c>
       <c r="O62" s="16" t="n">
         <v>841</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B63" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C63" s="16" t="n">
+        <v>190</v>
+      </c>
+      <c r="D63" s="16" t="n">
+        <v>4238</v>
+      </c>
+      <c r="E63" s="16" t="n">
+        <v>431</v>
+      </c>
+      <c r="F63" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G63" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="H63" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I63" s="16" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J63" s="16" t="n">
+        <v>128</v>
+      </c>
+      <c r="K63" s="16" t="n">
+        <v>1404</v>
+      </c>
+      <c r="L63" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="M63" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="N63" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O63" s="16" t="n">
+        <v>846</v>
       </c>
     </row>
   </sheetData>
@@ -6348,7 +6473,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9027,6 +9152,53 @@
       </c>
       <c r="O62" s="16" t="n">
         <v>327</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B63" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="C63" s="16" t="n">
+        <v>917</v>
+      </c>
+      <c r="D63" s="16" t="n">
+        <v>881</v>
+      </c>
+      <c r="E63" s="19" t="n">
+        <v>34.78</v>
+      </c>
+      <c r="F63" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G63" s="16" t="n">
+        <v>644</v>
+      </c>
+      <c r="H63" s="16" t="n">
+        <v>437</v>
+      </c>
+      <c r="I63" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="J63" s="19" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="K63" s="16" t="n">
+        <v>673</v>
+      </c>
+      <c r="L63" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="M63" s="16" t="n">
+        <v>69</v>
+      </c>
+      <c r="N63" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O63" s="16" t="n">
+        <v>313</v>
       </c>
     </row>
   </sheetData>
@@ -9045,7 +9217,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -11054,6 +11226,44 @@
         <v>270</v>
       </c>
       <c r="L59" s="16" t="n">
+        <v>241675</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B60" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C60" s="16" t="n">
+        <v>99</v>
+      </c>
+      <c r="D60" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E60" s="16" t="n">
+        <v>94</v>
+      </c>
+      <c r="F60" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G60" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H60" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I60" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J60" s="19" t="n">
+        <v>313.2</v>
+      </c>
+      <c r="K60" s="19" t="n">
+        <v>269.5</v>
+      </c>
+      <c r="L60" s="16" t="n">
         <v>241675</v>
       </c>
     </row>
@@ -11122,20 +11332,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>86</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11143,20 +11353,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>207</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>216</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11164,20 +11374,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>1507</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>1852</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11185,20 +11395,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>149</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>159</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11206,20 +11416,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>15</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11227,20 +11437,20 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>70</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>77</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11248,20 +11458,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H100,'Social — theo ngày'!$A$6:$A$100,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$100,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>750</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H103,'Social — theo ngày'!$A$6:$A$103,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$103,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>821</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11303,7 +11513,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B62</f>
+        <f aca="false">'Social — 28 ngày'!B63</f>
         <v>116</v>
       </c>
     </row>
@@ -11324,8 +11534,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C62</f>
-        <v>197</v>
+        <f aca="false">'Social — 28 ngày'!C63</f>
+        <v>190</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11345,8 +11555,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D62</f>
-        <v>4362</v>
+        <f aca="false">'Social — 28 ngày'!D63</f>
+        <v>4238</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11366,8 +11576,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E62</f>
-        <v>442</v>
+        <f aca="false">'Social — 28 ngày'!E63</f>
+        <v>431</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11387,7 +11597,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F62</f>
+        <f aca="false">'Social — 28 ngày'!F63</f>
         <v>49</v>
       </c>
     </row>
@@ -11408,8 +11618,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G62</f>
-        <v>37</v>
+        <f aca="false">'Social — 28 ngày'!G63</f>
+        <v>38</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11429,8 +11639,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H62</f>
-        <v>117</v>
+        <f aca="false">'Social — 28 ngày'!H63</f>
+        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11450,8 +11660,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I62</f>
-        <v>2466</v>
+        <f aca="false">'Social — 28 ngày'!I63</f>
+        <v>2250</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11471,8 +11681,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J62</f>
-        <v>124</v>
+        <f aca="false">'Social — 28 ngày'!J63</f>
+        <v>128</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11492,8 +11702,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K62</f>
-        <v>1243</v>
+        <f aca="false">'Social — 28 ngày'!K63</f>
+        <v>1404</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11513,8 +11723,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L62</f>
-        <v>30</v>
+        <f aca="false">'Social — 28 ngày'!L63</f>
+        <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11534,8 +11744,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M62</f>
-        <v>30</v>
+        <f aca="false">'Social — 28 ngày'!M63</f>
+        <v>44</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11555,7 +11765,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N62</f>
+        <f aca="false">'Social — 28 ngày'!N63</f>
         <v>7</v>
       </c>
     </row>
@@ -11576,8 +11786,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O62</f>
-        <v>841</v>
+        <f aca="false">'Social — 28 ngày'!O63</f>
+        <v>846</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11626,8 +11836,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B62</f>
-        <v>12</v>
+        <f aca="false">SEO!B63</f>
+        <v>13</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11651,7 +11861,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C62</f>
+        <f aca="false">SEO!C63</f>
         <v>917</v>
       </c>
     </row>
@@ -11676,7 +11886,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D62</f>
+        <f aca="false">SEO!D63</f>
         <v>881</v>
       </c>
     </row>
@@ -11701,8 +11911,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E62</f>
-        <v>34.02</v>
+        <f aca="false">SEO!E63</f>
+        <v>34.78</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11726,7 +11936,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F62</f>
+        <f aca="false">SEO!F63</f>
         <v>7</v>
       </c>
     </row>
@@ -11751,8 +11961,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G62</f>
-        <v>635</v>
+        <f aca="false">SEO!G63</f>
+        <v>644</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11776,8 +11986,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H62</f>
-        <v>440</v>
+        <f aca="false">SEO!H63</f>
+        <v>437</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11801,8 +12011,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I62</f>
-        <v>19</v>
+        <f aca="false">SEO!I63</f>
+        <v>22</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11826,8 +12036,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J62</f>
-        <v>2.8</v>
+        <f aca="false">SEO!J63</f>
+        <v>3.3</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11851,7 +12061,7 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K62</f>
+        <f aca="false">SEO!K63</f>
         <v>673</v>
       </c>
     </row>
@@ -11876,8 +12086,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L62</f>
-        <v>14.6</v>
+        <f aca="false">SEO!L63</f>
+        <v>12</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11901,8 +12111,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M62</f>
-        <v>78</v>
+        <f aca="false">SEO!M63</f>
+        <v>69</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11926,7 +12136,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N62</f>
+        <f aca="false">SEO!N63</f>
         <v>119</v>
       </c>
     </row>
@@ -11951,8 +12161,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O62</f>
-        <v>327</v>
+        <f aca="false">SEO!O63</f>
+        <v>313</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11994,7 +12204,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B59</f>
+        <f aca="false">Audit!B60</f>
         <v>93</v>
       </c>
     </row>
@@ -12015,8 +12225,8 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C59</f>
-        <v>98</v>
+        <f aca="false">Audit!C60</f>
+        <v>99</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12036,7 +12246,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D59</f>
+        <f aca="false">Audit!D60</f>
         <v>97</v>
       </c>
     </row>
@@ -12057,7 +12267,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E59</f>
+        <f aca="false">Audit!E60</f>
         <v>94</v>
       </c>
     </row>
@@ -12078,7 +12288,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F59</f>
+        <f aca="false">Audit!F60</f>
         <v>118</v>
       </c>
     </row>
@@ -12099,7 +12309,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G59</f>
+        <f aca="false">Audit!G60</f>
         <v>98</v>
       </c>
     </row>
@@ -12120,7 +12330,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H59</f>
+        <f aca="false">Audit!H60</f>
         <v>119</v>
       </c>
     </row>
@@ -12141,7 +12351,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I59</f>
+        <f aca="false">Audit!I60</f>
         <v>98</v>
       </c>
     </row>
@@ -12162,8 +12372,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J59</f>
-        <v>327</v>
+        <f aca="false">Audit!J60</f>
+        <v>313.2</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12183,8 +12393,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K59</f>
-        <v>270</v>
+        <f aca="false">Audit!K60</f>
+        <v>269.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12204,7 +12414,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L59</f>
+        <f aca="false">Audit!L60</f>
         <v>241675</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social: index 2026-10-14, hub weekly fallback, Excel
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-12 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-13 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">99 dòng × 7 chỉ số · 2026-07-05 → 2026-10-11</t>
+    <t xml:space="preserve">100 dòng × 7 chỉ số · 2026-07-05 → 2026-10-12</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">59 dòng × 14 chỉ số · 2026-07-23 → 2026-10-13</t>
+    <t xml:space="preserve">60 dòng × 14 chỉ số · 2026-07-23 → 2026-10-14</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">59 dòng × 14 chỉ số · 2026-06-30 → 2026-10-13</t>
+    <t xml:space="preserve">60 dòng × 14 chỉ số · 2026-06-30 → 2026-10-14</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">56 dòng × 11 chỉ số · 2026-07-27 → 2026-10-13</t>
+    <t xml:space="preserve">57 dòng × 11 chỉ số · 2026-07-27 → 2026-10-14</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 99 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 100 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 59 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 60 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 59 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 60 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 56 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 57 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3627,6 +3627,32 @@
       </c>
       <c r="H104" s="16" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B105" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C105" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="D105" s="16" t="n">
+        <v>201</v>
+      </c>
+      <c r="E105" s="16" t="n">
+        <v>82</v>
+      </c>
+      <c r="F105" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H105" s="16" t="n">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3645,7 +3671,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6527,6 +6553,53 @@
         <v>7</v>
       </c>
       <c r="O64" s="16" t="n">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B65" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C65" s="16" t="n">
+        <v>184</v>
+      </c>
+      <c r="D65" s="16" t="n">
+        <v>4139</v>
+      </c>
+      <c r="E65" s="16" t="n">
+        <v>493</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G65" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="H65" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="I65" s="16" t="n">
+        <v>2169</v>
+      </c>
+      <c r="J65" s="16" t="n">
+        <v>132</v>
+      </c>
+      <c r="K65" s="16" t="n">
+        <v>1090</v>
+      </c>
+      <c r="L65" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="M65" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="N65" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O65" s="16" t="n">
         <v>842</v>
       </c>
     </row>
@@ -6546,7 +6619,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9319,6 +9392,53 @@
       </c>
       <c r="O64" s="16" t="n">
         <v>316</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B65" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C65" s="16" t="n">
+        <v>915</v>
+      </c>
+      <c r="D65" s="16" t="n">
+        <v>879</v>
+      </c>
+      <c r="E65" s="19" t="n">
+        <v>36.76</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G65" s="16" t="n">
+        <v>672</v>
+      </c>
+      <c r="H65" s="16" t="n">
+        <v>448</v>
+      </c>
+      <c r="I65" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="J65" s="19" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K65" s="16" t="n">
+        <v>672</v>
+      </c>
+      <c r="L65" s="19" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="M65" s="16" t="n">
+        <v>67</v>
+      </c>
+      <c r="N65" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O65" s="16" t="n">
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -9337,7 +9457,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -11423,6 +11543,44 @@
       </c>
       <c r="L61" s="16" t="n">
         <v>242620</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B62" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C62" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D62" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E62" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="F62" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G62" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H62" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I62" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J62" s="19" t="n">
+        <v>317.4</v>
+      </c>
+      <c r="K62" s="19" t="n">
+        <v>267.5</v>
+      </c>
+      <c r="L62" s="16" t="n">
+        <v>241898</v>
       </c>
     </row>
   </sheetData>
@@ -11490,20 +11648,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>92</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11511,20 +11669,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>217</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>243</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11532,20 +11690,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>1886</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>2087</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11553,20 +11711,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>162</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11574,20 +11732,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>19</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11595,20 +11753,20 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>79</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11616,20 +11774,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H104,'Social — theo ngày'!$A$6:$A$104,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$104,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>830</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>959</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11671,7 +11829,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B64</f>
+        <f aca="false">'Social — 28 ngày'!B65</f>
         <v>116</v>
       </c>
     </row>
@@ -11692,8 +11850,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C64</f>
-        <v>190</v>
+        <f aca="false">'Social — 28 ngày'!C65</f>
+        <v>184</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11713,8 +11871,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D64</f>
-        <v>4156</v>
+        <f aca="false">'Social — 28 ngày'!D65</f>
+        <v>4139</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11734,8 +11892,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E64</f>
-        <v>418</v>
+        <f aca="false">'Social — 28 ngày'!E65</f>
+        <v>493</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11755,7 +11913,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F64</f>
+        <f aca="false">'Social — 28 ngày'!F65</f>
         <v>49</v>
       </c>
     </row>
@@ -11776,8 +11934,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G64</f>
-        <v>38</v>
+        <f aca="false">'Social — 28 ngày'!G65</f>
+        <v>39</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11797,8 +11955,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H64</f>
-        <v>119</v>
+        <f aca="false">'Social — 28 ngày'!H65</f>
+        <v>120</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11818,8 +11976,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I64</f>
-        <v>2218</v>
+        <f aca="false">'Social — 28 ngày'!I65</f>
+        <v>2169</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11839,8 +11997,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J64</f>
-        <v>131</v>
+        <f aca="false">'Social — 28 ngày'!J65</f>
+        <v>132</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11860,8 +12018,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K64</f>
-        <v>1103</v>
+        <f aca="false">'Social — 28 ngày'!K65</f>
+        <v>1090</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11881,8 +12039,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L64</f>
-        <v>58</v>
+        <f aca="false">'Social — 28 ngày'!L65</f>
+        <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11902,7 +12060,7 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M64</f>
+        <f aca="false">'Social — 28 ngày'!M65</f>
         <v>41</v>
       </c>
     </row>
@@ -11923,7 +12081,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N64</f>
+        <f aca="false">'Social — 28 ngày'!N65</f>
         <v>7</v>
       </c>
     </row>
@@ -11944,7 +12102,7 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O64</f>
+        <f aca="false">'Social — 28 ngày'!O65</f>
         <v>842</v>
       </c>
     </row>
@@ -11994,7 +12152,7 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B64</f>
+        <f aca="false">SEO!B65</f>
         <v>14</v>
       </c>
     </row>
@@ -12019,8 +12177,8 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C64</f>
-        <v>917</v>
+        <f aca="false">SEO!C65</f>
+        <v>915</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12044,8 +12202,8 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D64</f>
-        <v>881</v>
+        <f aca="false">SEO!D65</f>
+        <v>879</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12069,8 +12227,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E64</f>
-        <v>35.91</v>
+        <f aca="false">SEO!E65</f>
+        <v>36.76</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12094,7 +12252,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F64</f>
+        <f aca="false">SEO!F65</f>
         <v>7</v>
       </c>
     </row>
@@ -12119,8 +12277,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G64</f>
-        <v>660</v>
+        <f aca="false">SEO!G65</f>
+        <v>672</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12144,8 +12302,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H64</f>
-        <v>443</v>
+        <f aca="false">SEO!H65</f>
+        <v>448</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12169,8 +12327,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I64</f>
-        <v>24</v>
+        <f aca="false">SEO!I65</f>
+        <v>23</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12194,8 +12352,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J64</f>
-        <v>3.6</v>
+        <f aca="false">SEO!J65</f>
+        <v>3.4</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12219,8 +12377,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K64</f>
-        <v>673</v>
+        <f aca="false">SEO!K65</f>
+        <v>672</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12244,8 +12402,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L64</f>
-        <v>12</v>
+        <f aca="false">SEO!L65</f>
+        <v>12.1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12269,8 +12427,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M64</f>
-        <v>68</v>
+        <f aca="false">SEO!M65</f>
+        <v>67</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12294,7 +12452,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N64</f>
+        <f aca="false">SEO!N65</f>
         <v>119</v>
       </c>
     </row>
@@ -12319,8 +12477,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O64</f>
-        <v>316</v>
+        <f aca="false">SEO!O65</f>
+        <v>317</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12362,7 +12520,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B61</f>
+        <f aca="false">Audit!B62</f>
         <v>93</v>
       </c>
     </row>
@@ -12383,7 +12541,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C61</f>
+        <f aca="false">Audit!C62</f>
         <v>98</v>
       </c>
     </row>
@@ -12404,7 +12562,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D61</f>
+        <f aca="false">Audit!D62</f>
         <v>97</v>
       </c>
     </row>
@@ -12425,8 +12583,8 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E61</f>
-        <v>94</v>
+        <f aca="false">Audit!E62</f>
+        <v>93</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12446,7 +12604,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F61</f>
+        <f aca="false">Audit!F62</f>
         <v>118</v>
       </c>
     </row>
@@ -12467,7 +12625,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G61</f>
+        <f aca="false">Audit!G62</f>
         <v>98</v>
       </c>
     </row>
@@ -12488,7 +12646,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H61</f>
+        <f aca="false">Audit!H62</f>
         <v>119</v>
       </c>
     </row>
@@ -12509,7 +12667,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I61</f>
+        <f aca="false">Audit!I62</f>
         <v>98</v>
       </c>
     </row>
@@ -12530,8 +12688,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J61</f>
-        <v>315.9</v>
+        <f aca="false">Audit!J62</f>
+        <v>317.4</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12551,8 +12709,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K61</f>
-        <v>261</v>
+        <f aca="false">Audit!K62</f>
+        <v>267.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12572,8 +12730,8 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L61</f>
-        <v>242620</v>
+        <f aca="false">Audit!L62</f>
+        <v>241898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Social: index.html + dxl-metrics.xlsx 2026-10-15
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-13 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-14 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">100 dòng × 7 chỉ số · 2026-07-05 → 2026-10-12</t>
+    <t xml:space="preserve">101 dòng × 7 chỉ số · 2026-07-05 → 2026-10-13</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">60 dòng × 14 chỉ số · 2026-07-23 → 2026-10-14</t>
+    <t xml:space="preserve">61 dòng × 14 chỉ số · 2026-07-23 → 2026-10-15</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">60 dòng × 14 chỉ số · 2026-06-30 → 2026-10-14</t>
+    <t xml:space="preserve">61 dòng × 14 chỉ số · 2026-06-30 → 2026-10-15</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">57 dòng × 11 chỉ số · 2026-07-27 → 2026-10-14</t>
+    <t xml:space="preserve">58 dòng × 11 chỉ số · 2026-07-27 → 2026-10-15</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 100 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 101 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 60 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 61 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 60 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 61 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 57 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 58 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3653,6 +3653,32 @@
       </c>
       <c r="H105" s="16" t="n">
         <v>129</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B106" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C106" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="16" t="n">
+        <v>71</v>
+      </c>
+      <c r="E106" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="F106" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" s="16" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3671,7 +3697,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6601,6 +6627,53 @@
       </c>
       <c r="O65" s="16" t="n">
         <v>842</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B66" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C66" s="16" t="n">
+        <v>181</v>
+      </c>
+      <c r="D66" s="16" t="n">
+        <v>3995</v>
+      </c>
+      <c r="E66" s="16" t="n">
+        <v>432</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G66" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="H66" s="16" t="n">
+        <v>85</v>
+      </c>
+      <c r="I66" s="16" t="n">
+        <v>1868</v>
+      </c>
+      <c r="J66" s="16" t="n">
+        <v>133</v>
+      </c>
+      <c r="K66" s="16" t="n">
+        <v>1108</v>
+      </c>
+      <c r="L66" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="M66" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="N66" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O66" s="16" t="n">
+        <v>721</v>
       </c>
     </row>
   </sheetData>
@@ -6619,7 +6692,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9439,6 +9512,53 @@
       </c>
       <c r="O65" s="16" t="n">
         <v>317</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B66" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C66" s="16" t="n">
+        <v>913</v>
+      </c>
+      <c r="D66" s="16" t="n">
+        <v>877</v>
+      </c>
+      <c r="E66" s="19" t="n">
+        <v>37.77</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="G66" s="16" t="n">
+        <v>683</v>
+      </c>
+      <c r="H66" s="16" t="n">
+        <v>454</v>
+      </c>
+      <c r="I66" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="J66" s="19" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K66" s="16" t="n">
+        <v>730</v>
+      </c>
+      <c r="L66" s="19" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="M66" s="16" t="n">
+        <v>76</v>
+      </c>
+      <c r="N66" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O66" s="16" t="n">
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -9457,7 +9577,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -11581,6 +11701,44 @@
       </c>
       <c r="L62" s="16" t="n">
         <v>241898</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B63" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C63" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D63" s="16" t="n">
+        <v>96</v>
+      </c>
+      <c r="E63" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="F63" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G63" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="H63" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I63" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J63" s="19" t="n">
+        <v>324.9</v>
+      </c>
+      <c r="K63" s="16" t="n">
+        <v>269</v>
+      </c>
+      <c r="L63" s="16" t="n">
+        <v>242263</v>
       </c>
     </row>
   </sheetData>
@@ -11648,20 +11806,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>94</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11669,20 +11827,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>243</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>244</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11690,20 +11848,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>2087</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>2158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11711,20 +11869,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>244</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11732,19 +11890,19 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>20</v>
       </c>
     </row>
@@ -11753,19 +11911,19 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>85</v>
       </c>
     </row>
@@ -11774,20 +11932,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H105,'Social — theo ngày'!$A$6:$A$105,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$105,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>959</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H106,'Social — theo ngày'!$A$6:$A$106,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$106,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>968</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11829,7 +11987,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B65</f>
+        <f aca="false">'Social — 28 ngày'!B66</f>
         <v>116</v>
       </c>
     </row>
@@ -11850,8 +12008,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C65</f>
-        <v>184</v>
+        <f aca="false">'Social — 28 ngày'!C66</f>
+        <v>181</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11871,8 +12029,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D65</f>
-        <v>4139</v>
+        <f aca="false">'Social — 28 ngày'!D66</f>
+        <v>3995</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11892,8 +12050,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E65</f>
-        <v>493</v>
+        <f aca="false">'Social — 28 ngày'!E66</f>
+        <v>432</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11913,7 +12071,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F65</f>
+        <f aca="false">'Social — 28 ngày'!F66</f>
         <v>49</v>
       </c>
     </row>
@@ -11934,8 +12092,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G65</f>
-        <v>39</v>
+        <f aca="false">'Social — 28 ngày'!G66</f>
+        <v>36</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11955,8 +12113,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H65</f>
-        <v>120</v>
+        <f aca="false">'Social — 28 ngày'!H66</f>
+        <v>85</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11976,8 +12134,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I65</f>
-        <v>2169</v>
+        <f aca="false">'Social — 28 ngày'!I66</f>
+        <v>1868</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11997,8 +12155,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J65</f>
-        <v>132</v>
+        <f aca="false">'Social — 28 ngày'!J66</f>
+        <v>133</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12018,8 +12176,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K65</f>
-        <v>1090</v>
+        <f aca="false">'Social — 28 ngày'!K66</f>
+        <v>1108</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12039,8 +12197,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L65</f>
-        <v>59</v>
+        <f aca="false">'Social — 28 ngày'!L66</f>
+        <v>60</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12060,8 +12218,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M65</f>
-        <v>41</v>
+        <f aca="false">'Social — 28 ngày'!M66</f>
+        <v>37</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12081,7 +12239,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N65</f>
+        <f aca="false">'Social — 28 ngày'!N66</f>
         <v>7</v>
       </c>
     </row>
@@ -12102,8 +12260,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O65</f>
-        <v>842</v>
+        <f aca="false">'Social — 28 ngày'!O66</f>
+        <v>721</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12152,7 +12310,7 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B65</f>
+        <f aca="false">SEO!B66</f>
         <v>14</v>
       </c>
     </row>
@@ -12177,8 +12335,8 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C65</f>
-        <v>915</v>
+        <f aca="false">SEO!C66</f>
+        <v>913</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12202,8 +12360,8 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D65</f>
-        <v>879</v>
+        <f aca="false">SEO!D66</f>
+        <v>877</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12227,8 +12385,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E65</f>
-        <v>36.76</v>
+        <f aca="false">SEO!E66</f>
+        <v>37.77</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12252,8 +12410,8 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F65</f>
-        <v>7</v>
+        <f aca="false">SEO!F66</f>
+        <v>9</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12277,8 +12435,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G65</f>
-        <v>672</v>
+        <f aca="false">SEO!G66</f>
+        <v>683</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12302,8 +12460,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H65</f>
-        <v>448</v>
+        <f aca="false">SEO!H66</f>
+        <v>454</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12327,8 +12485,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I65</f>
-        <v>23</v>
+        <f aca="false">SEO!I66</f>
+        <v>25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12352,7 +12510,7 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J65</f>
+        <f aca="false">SEO!J66</f>
         <v>3.4</v>
       </c>
     </row>
@@ -12377,8 +12535,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K65</f>
-        <v>672</v>
+        <f aca="false">SEO!K66</f>
+        <v>730</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12402,8 +12560,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L65</f>
-        <v>12.1</v>
+        <f aca="false">SEO!L66</f>
+        <v>12.3</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12427,8 +12585,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M65</f>
-        <v>67</v>
+        <f aca="false">SEO!M66</f>
+        <v>76</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12452,7 +12610,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N65</f>
+        <f aca="false">SEO!N66</f>
         <v>119</v>
       </c>
     </row>
@@ -12477,8 +12635,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O65</f>
-        <v>317</v>
+        <f aca="false">SEO!O66</f>
+        <v>325</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12520,7 +12678,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B62</f>
+        <f aca="false">Audit!B63</f>
         <v>93</v>
       </c>
     </row>
@@ -12541,7 +12699,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C62</f>
+        <f aca="false">Audit!C63</f>
         <v>98</v>
       </c>
     </row>
@@ -12562,8 +12720,8 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D62</f>
-        <v>97</v>
+        <f aca="false">Audit!D63</f>
+        <v>96</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12583,7 +12741,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E62</f>
+        <f aca="false">Audit!E63</f>
         <v>93</v>
       </c>
     </row>
@@ -12604,7 +12762,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F62</f>
+        <f aca="false">Audit!F63</f>
         <v>118</v>
       </c>
     </row>
@@ -12625,8 +12783,8 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G62</f>
-        <v>98</v>
+        <f aca="false">Audit!G63</f>
+        <v>97</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12646,7 +12804,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H62</f>
+        <f aca="false">Audit!H63</f>
         <v>119</v>
       </c>
     </row>
@@ -12667,7 +12825,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I62</f>
+        <f aca="false">Audit!I63</f>
         <v>98</v>
       </c>
     </row>
@@ -12688,8 +12846,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J62</f>
-        <v>317.4</v>
+        <f aca="false">Audit!J63</f>
+        <v>324.9</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12709,8 +12867,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K62</f>
-        <v>267.5</v>
+        <f aca="false">Audit!K63</f>
+        <v>269</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12730,8 +12888,8 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L62</f>
-        <v>241898</v>
+        <f aca="false">Audit!L63</f>
+        <v>242263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Social: index.html + dxl-metrics.xlsx 2026-10-20
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-17 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-19 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">104 dòng × 7 chỉ số · 2026-07-05 → 2026-10-16</t>
+    <t xml:space="preserve">106 dòng × 7 chỉ số · 2026-07-05 → 2026-10-18</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">63 dòng × 14 chỉ số · 2026-07-23 → 2026-10-18</t>
+    <t xml:space="preserve">64 dòng × 14 chỉ số · 2026-07-23 → 2026-10-20</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">63 dòng × 14 chỉ số · 2026-06-30 → 2026-10-18</t>
+    <t xml:space="preserve">64 dòng × 14 chỉ số · 2026-06-30 → 2026-10-20</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">60 dòng × 11 chỉ số · 2026-07-27 → 2026-10-18</t>
+    <t xml:space="preserve">61 dòng × 11 chỉ số · 2026-07-27 → 2026-10-20</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 104 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 106 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 63 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 64 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 63 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 64 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 60 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 61 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3751,6 +3751,54 @@
       <c r="G109" s="16"/>
       <c r="H109" s="16" t="n">
         <v>24</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="15" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B110" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C110" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="D110" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="E110" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F110" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" s="16"/>
+      <c r="H110" s="16" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="15" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B111" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="D111" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="E111" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="F111" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G111" s="16"/>
+      <c r="H111" s="16" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -3769,7 +3817,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O68"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6832,6 +6880,53 @@
       </c>
       <c r="O68" s="16" t="n">
         <v>586</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B69" s="16" t="n">
+        <v>117</v>
+      </c>
+      <c r="C69" s="16" t="n">
+        <v>173</v>
+      </c>
+      <c r="D69" s="16" t="n">
+        <v>3981</v>
+      </c>
+      <c r="E69" s="16" t="n">
+        <v>490</v>
+      </c>
+      <c r="F69" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G69" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="H69" s="16" t="n">
+        <v>285</v>
+      </c>
+      <c r="I69" s="16" t="n">
+        <v>1775</v>
+      </c>
+      <c r="J69" s="16" t="n">
+        <v>138</v>
+      </c>
+      <c r="K69" s="16" t="n">
+        <v>1278</v>
+      </c>
+      <c r="L69" s="16" t="n">
+        <v>82</v>
+      </c>
+      <c r="M69" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="N69" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O69" s="16" t="n">
+        <v>780</v>
       </c>
     </row>
   </sheetData>
@@ -6850,7 +6945,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O68"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9811,6 +9906,53 @@
       </c>
       <c r="O68" s="16" t="n">
         <v>325</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B69" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="C69" s="16" t="n">
+        <v>912</v>
+      </c>
+      <c r="D69" s="16" t="n">
+        <v>876</v>
+      </c>
+      <c r="E69" s="19" t="n">
+        <v>40.27</v>
+      </c>
+      <c r="F69" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="G69" s="16" t="n">
+        <v>673</v>
+      </c>
+      <c r="H69" s="16" t="n">
+        <v>425</v>
+      </c>
+      <c r="I69" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="J69" s="19" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="K69" s="16" t="n">
+        <v>951</v>
+      </c>
+      <c r="L69" s="19" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="M69" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="N69" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O69" s="16" t="n">
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -9829,7 +9971,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -12066,6 +12208,44 @@
         <v>266.5</v>
       </c>
       <c r="L65" s="16" t="n">
+        <v>242263</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B66" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C66" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D66" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E66" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G66" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H66" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I66" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J66" s="19" t="n">
+        <v>301.8</v>
+      </c>
+      <c r="K66" s="16" t="n">
+        <v>247</v>
+      </c>
+      <c r="L66" s="16" t="n">
         <v>242263</v>
       </c>
     </row>
@@ -12134,20 +12314,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>108</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>112</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12155,20 +12335,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>282</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>326</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12176,20 +12356,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>2543</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>2704</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12197,20 +12377,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>355</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>398</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12218,20 +12398,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>27</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>28</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12239,19 +12419,19 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>85</v>
       </c>
     </row>
@@ -12260,20 +12440,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H109,'Social — theo ngày'!$A$6:$A$109,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$109,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>1190</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>1336</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12315,8 +12495,8 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B68</f>
-        <v>116</v>
+        <f aca="false">'Social — 28 ngày'!B69</f>
+        <v>117</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12336,8 +12516,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C68</f>
-        <v>171</v>
+        <f aca="false">'Social — 28 ngày'!C69</f>
+        <v>173</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12357,8 +12537,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D68</f>
-        <v>3891</v>
+        <f aca="false">'Social — 28 ngày'!D69</f>
+        <v>3981</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12378,8 +12558,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E68</f>
-        <v>462</v>
+        <f aca="false">'Social — 28 ngày'!E69</f>
+        <v>490</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12399,7 +12579,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F68</f>
+        <f aca="false">'Social — 28 ngày'!F69</f>
         <v>49</v>
       </c>
     </row>
@@ -12420,8 +12600,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G68</f>
-        <v>43</v>
+        <f aca="false">'Social — 28 ngày'!G69</f>
+        <v>44</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12441,8 +12621,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H68</f>
-        <v>175</v>
+        <f aca="false">'Social — 28 ngày'!H69</f>
+        <v>285</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12462,8 +12642,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I68</f>
-        <v>1665</v>
+        <f aca="false">'Social — 28 ngày'!I69</f>
+        <v>1775</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12483,8 +12663,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J68</f>
-        <v>136</v>
+        <f aca="false">'Social — 28 ngày'!J69</f>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12504,8 +12684,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K68</f>
-        <v>1299</v>
+        <f aca="false">'Social — 28 ngày'!K69</f>
+        <v>1278</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12525,8 +12705,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L68</f>
-        <v>79</v>
+        <f aca="false">'Social — 28 ngày'!L69</f>
+        <v>82</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12546,8 +12726,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M68</f>
-        <v>38</v>
+        <f aca="false">'Social — 28 ngày'!M69</f>
+        <v>37</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12567,7 +12747,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N68</f>
+        <f aca="false">'Social — 28 ngày'!N69</f>
         <v>7</v>
       </c>
     </row>
@@ -12588,8 +12768,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O68</f>
-        <v>586</v>
+        <f aca="false">'Social — 28 ngày'!O69</f>
+        <v>780</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12638,8 +12818,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B68</f>
-        <v>17</v>
+        <f aca="false">SEO!B69</f>
+        <v>18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12663,7 +12843,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C68</f>
+        <f aca="false">SEO!C69</f>
         <v>912</v>
       </c>
     </row>
@@ -12688,7 +12868,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D68</f>
+        <f aca="false">SEO!D69</f>
         <v>876</v>
       </c>
     </row>
@@ -12713,8 +12893,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E68</f>
-        <v>39.18</v>
+        <f aca="false">SEO!E69</f>
+        <v>40.27</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12738,7 +12918,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F68</f>
+        <f aca="false">SEO!F69</f>
         <v>9</v>
       </c>
     </row>
@@ -12763,8 +12943,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G68</f>
-        <v>679</v>
+        <f aca="false">SEO!G69</f>
+        <v>673</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12788,8 +12968,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H68</f>
-        <v>433</v>
+        <f aca="false">SEO!H69</f>
+        <v>425</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12813,7 +12993,7 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I68</f>
+        <f aca="false">SEO!I69</f>
         <v>26</v>
       </c>
     </row>
@@ -12838,8 +13018,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J68</f>
-        <v>3.2</v>
+        <f aca="false">SEO!J69</f>
+        <v>2.7</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12863,8 +13043,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K68</f>
-        <v>816</v>
+        <f aca="false">SEO!K69</f>
+        <v>951</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12888,8 +13068,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L68</f>
-        <v>15.2</v>
+        <f aca="false">SEO!L69</f>
+        <v>17.6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12913,8 +13093,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M68</f>
-        <v>83</v>
+        <f aca="false">SEO!M69</f>
+        <v>90</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12938,7 +13118,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N68</f>
+        <f aca="false">SEO!N69</f>
         <v>119</v>
       </c>
     </row>
@@ -12963,8 +13143,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O68</f>
-        <v>325</v>
+        <f aca="false">SEO!O69</f>
+        <v>302</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13006,7 +13186,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B65</f>
+        <f aca="false">Audit!B66</f>
         <v>93</v>
       </c>
     </row>
@@ -13027,7 +13207,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C65</f>
+        <f aca="false">Audit!C66</f>
         <v>98</v>
       </c>
     </row>
@@ -13048,7 +13228,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D65</f>
+        <f aca="false">Audit!D66</f>
         <v>97</v>
       </c>
     </row>
@@ -13069,7 +13249,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E65</f>
+        <f aca="false">Audit!E66</f>
         <v>93</v>
       </c>
     </row>
@@ -13090,7 +13270,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F65</f>
+        <f aca="false">Audit!F66</f>
         <v>118</v>
       </c>
     </row>
@@ -13111,7 +13291,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G65</f>
+        <f aca="false">Audit!G66</f>
         <v>98</v>
       </c>
     </row>
@@ -13132,7 +13312,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H65</f>
+        <f aca="false">Audit!H66</f>
         <v>119</v>
       </c>
     </row>
@@ -13153,7 +13333,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I65</f>
+        <f aca="false">Audit!I66</f>
         <v>98</v>
       </c>
     </row>
@@ -13174,8 +13354,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J65</f>
-        <v>324.9</v>
+        <f aca="false">Audit!J66</f>
+        <v>301.8</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13195,8 +13375,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K65</f>
-        <v>266.5</v>
+        <f aca="false">Audit!K66</f>
+        <v>247</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13216,7 +13396,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L65</f>
+        <f aca="false">Audit!L66</f>
         <v>242263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social: index.html + dxl-metrics.xlsx 2026-10-21
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-19 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-20 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">106 dòng × 7 chỉ số · 2026-07-05 → 2026-10-18</t>
+    <t xml:space="preserve">107 dòng × 7 chỉ số · 2026-07-05 → 2026-10-19</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">64 dòng × 14 chỉ số · 2026-07-23 → 2026-10-20</t>
+    <t xml:space="preserve">65 dòng × 14 chỉ số · 2026-07-23 → 2026-10-21</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">64 dòng × 14 chỉ số · 2026-06-30 → 2026-10-20</t>
+    <t xml:space="preserve">65 dòng × 14 chỉ số · 2026-06-30 → 2026-10-21</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">61 dòng × 11 chỉ số · 2026-07-27 → 2026-10-20</t>
+    <t xml:space="preserve">62 dòng × 11 chỉ số · 2026-07-27 → 2026-10-21</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 106 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 107 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 64 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 65 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 64 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 65 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 61 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 62 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3799,6 +3799,30 @@
       <c r="G111" s="16"/>
       <c r="H111" s="16" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B112" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C112" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D112" s="16" t="n">
+        <v>125</v>
+      </c>
+      <c r="E112" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="F112" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G112" s="16"/>
+      <c r="H112" s="16" t="n">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -3817,7 +3841,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6927,6 +6951,53 @@
       </c>
       <c r="O69" s="16" t="n">
         <v>780</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B70" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C70" s="16" t="n">
+        <v>171</v>
+      </c>
+      <c r="D70" s="16" t="n">
+        <v>3957</v>
+      </c>
+      <c r="E70" s="16" t="n">
+        <v>499</v>
+      </c>
+      <c r="F70" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G70" s="16" t="n">
+        <v>48</v>
+      </c>
+      <c r="H70" s="16" t="n">
+        <v>286</v>
+      </c>
+      <c r="I70" s="16" t="n">
+        <v>1767</v>
+      </c>
+      <c r="J70" s="16" t="n">
+        <v>139</v>
+      </c>
+      <c r="K70" s="16" t="n">
+        <v>1263</v>
+      </c>
+      <c r="L70" s="16" t="n">
+        <v>80</v>
+      </c>
+      <c r="M70" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="N70" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O70" s="16" t="n">
+        <v>782</v>
       </c>
     </row>
   </sheetData>
@@ -6945,7 +7016,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -9953,6 +10024,53 @@
       </c>
       <c r="O69" s="16" t="n">
         <v>302</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B70" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="C70" s="16" t="n">
+        <v>911</v>
+      </c>
+      <c r="D70" s="16" t="n">
+        <v>875</v>
+      </c>
+      <c r="E70" s="19" t="n">
+        <v>40.36</v>
+      </c>
+      <c r="F70" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="G70" s="16" t="n">
+        <v>669</v>
+      </c>
+      <c r="H70" s="16" t="n">
+        <v>419</v>
+      </c>
+      <c r="I70" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="J70" s="19" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K70" s="16" t="n">
+        <v>1017</v>
+      </c>
+      <c r="L70" s="19" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="M70" s="16" t="n">
+        <v>110</v>
+      </c>
+      <c r="N70" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O70" s="16" t="n">
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -9971,7 +10089,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -12246,6 +12364,44 @@
         <v>247</v>
       </c>
       <c r="L66" s="16" t="n">
+        <v>242263</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B67" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C67" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D67" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E67" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="F67" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G67" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H67" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I67" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J67" s="16" t="n">
+        <v>308</v>
+      </c>
+      <c r="K67" s="16" t="n">
+        <v>253</v>
+      </c>
+      <c r="L67" s="16" t="n">
         <v>242263</v>
       </c>
     </row>
@@ -12314,20 +12470,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>112</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12335,20 +12491,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>326</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>328</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12356,20 +12512,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>2704</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>2829</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12377,20 +12533,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>398</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>419</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12398,20 +12554,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>28</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>32</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12419,19 +12575,19 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>85</v>
       </c>
     </row>
@@ -12440,20 +12596,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H111,'Social — theo ngày'!$A$6:$A$111,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$111,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>1336</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>1385</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12495,8 +12651,8 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B69</f>
-        <v>117</v>
+        <f aca="false">'Social — 28 ngày'!B70</f>
+        <v>116</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12516,8 +12672,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C69</f>
-        <v>173</v>
+        <f aca="false">'Social — 28 ngày'!C70</f>
+        <v>171</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12537,8 +12693,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D69</f>
-        <v>3981</v>
+        <f aca="false">'Social — 28 ngày'!D70</f>
+        <v>3957</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12558,8 +12714,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E69</f>
-        <v>490</v>
+        <f aca="false">'Social — 28 ngày'!E70</f>
+        <v>499</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12579,7 +12735,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F69</f>
+        <f aca="false">'Social — 28 ngày'!F70</f>
         <v>49</v>
       </c>
     </row>
@@ -12600,8 +12756,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G69</f>
-        <v>44</v>
+        <f aca="false">'Social — 28 ngày'!G70</f>
+        <v>48</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12621,8 +12777,8 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H69</f>
-        <v>285</v>
+        <f aca="false">'Social — 28 ngày'!H70</f>
+        <v>286</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12642,8 +12798,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I69</f>
-        <v>1775</v>
+        <f aca="false">'Social — 28 ngày'!I70</f>
+        <v>1767</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12663,8 +12819,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J69</f>
-        <v>138</v>
+        <f aca="false">'Social — 28 ngày'!J70</f>
+        <v>139</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12684,8 +12840,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K69</f>
-        <v>1278</v>
+        <f aca="false">'Social — 28 ngày'!K70</f>
+        <v>1263</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12705,8 +12861,8 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L69</f>
-        <v>82</v>
+        <f aca="false">'Social — 28 ngày'!L70</f>
+        <v>80</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12726,8 +12882,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M69</f>
-        <v>37</v>
+        <f aca="false">'Social — 28 ngày'!M70</f>
+        <v>38</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12747,7 +12903,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N69</f>
+        <f aca="false">'Social — 28 ngày'!N70</f>
         <v>7</v>
       </c>
     </row>
@@ -12768,8 +12924,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O69</f>
-        <v>780</v>
+        <f aca="false">'Social — 28 ngày'!O70</f>
+        <v>782</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12818,8 +12974,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B69</f>
-        <v>18</v>
+        <f aca="false">SEO!B70</f>
+        <v>19</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12843,8 +12999,8 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C69</f>
-        <v>912</v>
+        <f aca="false">SEO!C70</f>
+        <v>911</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12868,8 +13024,8 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D69</f>
-        <v>876</v>
+        <f aca="false">SEO!D70</f>
+        <v>875</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12893,8 +13049,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E69</f>
-        <v>40.27</v>
+        <f aca="false">SEO!E70</f>
+        <v>40.36</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12918,7 +13074,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F69</f>
+        <f aca="false">SEO!F70</f>
         <v>9</v>
       </c>
     </row>
@@ -12943,8 +13099,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G69</f>
-        <v>673</v>
+        <f aca="false">SEO!G70</f>
+        <v>669</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12968,8 +13124,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H69</f>
-        <v>425</v>
+        <f aca="false">SEO!H70</f>
+        <v>419</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12993,8 +13149,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I69</f>
-        <v>26</v>
+        <f aca="false">SEO!I70</f>
+        <v>28</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13018,8 +13174,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J69</f>
-        <v>2.7</v>
+        <f aca="false">SEO!J70</f>
+        <v>2.8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13043,8 +13199,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K69</f>
-        <v>951</v>
+        <f aca="false">SEO!K70</f>
+        <v>1017</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13068,8 +13224,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L69</f>
-        <v>17.6</v>
+        <f aca="false">SEO!L70</f>
+        <v>19.1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13093,8 +13249,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M69</f>
-        <v>90</v>
+        <f aca="false">SEO!M70</f>
+        <v>110</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13118,7 +13274,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N69</f>
+        <f aca="false">SEO!N70</f>
         <v>119</v>
       </c>
     </row>
@@ -13143,8 +13299,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O69</f>
-        <v>302</v>
+        <f aca="false">SEO!O70</f>
+        <v>308</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13186,7 +13342,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B66</f>
+        <f aca="false">Audit!B67</f>
         <v>93</v>
       </c>
     </row>
@@ -13207,7 +13363,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C66</f>
+        <f aca="false">Audit!C67</f>
         <v>98</v>
       </c>
     </row>
@@ -13228,7 +13384,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D66</f>
+        <f aca="false">Audit!D67</f>
         <v>97</v>
       </c>
     </row>
@@ -13249,7 +13405,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E66</f>
+        <f aca="false">Audit!E67</f>
         <v>93</v>
       </c>
     </row>
@@ -13270,7 +13426,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F66</f>
+        <f aca="false">Audit!F67</f>
         <v>118</v>
       </c>
     </row>
@@ -13291,7 +13447,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G66</f>
+        <f aca="false">Audit!G67</f>
         <v>98</v>
       </c>
     </row>
@@ -13312,7 +13468,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H66</f>
+        <f aca="false">Audit!H67</f>
         <v>119</v>
       </c>
     </row>
@@ -13333,7 +13489,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I66</f>
+        <f aca="false">Audit!I67</f>
         <v>98</v>
       </c>
     </row>
@@ -13354,8 +13510,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J66</f>
-        <v>301.8</v>
+        <f aca="false">Audit!J67</f>
+        <v>308</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13375,8 +13531,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K66</f>
-        <v>247</v>
+        <f aca="false">Audit!K67</f>
+        <v>253</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13396,7 +13552,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L66</f>
+        <f aca="false">Audit!L67</f>
         <v>242263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Social: index.html + dxl-metrics.xlsx 2026-10-22
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-20 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-21 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">107 dòng × 7 chỉ số · 2026-07-05 → 2026-10-19</t>
+    <t xml:space="preserve">108 dòng × 7 chỉ số · 2026-07-05 → 2026-10-20</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">65 dòng × 14 chỉ số · 2026-07-23 → 2026-10-21</t>
+    <t xml:space="preserve">66 dòng × 14 chỉ số · 2026-07-23 → 2026-10-22</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">65 dòng × 14 chỉ số · 2026-06-30 → 2026-10-21</t>
+    <t xml:space="preserve">66 dòng × 14 chỉ số · 2026-06-30 → 2026-10-22</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">62 dòng × 11 chỉ số · 2026-07-27 → 2026-10-21</t>
+    <t xml:space="preserve">63 dòng × 11 chỉ số · 2026-07-27 → 2026-10-22</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 107 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 108 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 65 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 66 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 65 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 66 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 62 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 63 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3823,6 +3823,30 @@
       <c r="G112" s="16"/>
       <c r="H112" s="16" t="n">
         <v>49</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B113" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C113" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D113" s="16" t="n">
+        <v>203</v>
+      </c>
+      <c r="E113" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="F113" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="G113" s="16"/>
+      <c r="H113" s="16" t="n">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -3841,7 +3865,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6998,6 +7022,53 @@
       </c>
       <c r="O70" s="16" t="n">
         <v>782</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B71" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="C71" s="16" t="n">
+        <v>177</v>
+      </c>
+      <c r="D71" s="16" t="n">
+        <v>4026</v>
+      </c>
+      <c r="E71" s="16" t="n">
+        <v>517</v>
+      </c>
+      <c r="F71" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="G71" s="16" t="n">
+        <v>57</v>
+      </c>
+      <c r="H71" s="16" t="n">
+        <v>286</v>
+      </c>
+      <c r="I71" s="16" t="n">
+        <v>1790</v>
+      </c>
+      <c r="J71" s="16" t="n">
+        <v>138</v>
+      </c>
+      <c r="K71" s="16" t="n">
+        <v>1250</v>
+      </c>
+      <c r="L71" s="16" t="n">
+        <v>80</v>
+      </c>
+      <c r="M71" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="N71" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O71" s="16" t="n">
+        <v>783</v>
       </c>
     </row>
   </sheetData>
@@ -7016,7 +7087,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -10071,6 +10142,53 @@
       </c>
       <c r="O70" s="16" t="n">
         <v>308</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B71" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="C71" s="16" t="n">
+        <v>911</v>
+      </c>
+      <c r="D71" s="16" t="n">
+        <v>875</v>
+      </c>
+      <c r="E71" s="19" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="F71" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G71" s="16" t="n">
+        <v>672</v>
+      </c>
+      <c r="H71" s="16" t="n">
+        <v>422</v>
+      </c>
+      <c r="I71" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="J71" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K71" s="16" t="n">
+        <v>1174</v>
+      </c>
+      <c r="L71" s="19" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="M71" s="16" t="n">
+        <v>114</v>
+      </c>
+      <c r="N71" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="O71" s="19" t="n">
+        <v>311.2</v>
       </c>
     </row>
   </sheetData>
@@ -10089,7 +10207,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -12403,6 +12521,44 @@
       </c>
       <c r="L67" s="16" t="n">
         <v>242263</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B68" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C68" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D68" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E68" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="F68" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="G68" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="H68" s="16" t="n">
+        <v>119</v>
+      </c>
+      <c r="I68" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J68" s="19" t="n">
+        <v>311.2</v>
+      </c>
+      <c r="K68" s="16" t="n">
+        <v>255</v>
+      </c>
+      <c r="L68" s="16" t="n">
+        <v>243021</v>
       </c>
     </row>
   </sheetData>
@@ -12470,20 +12626,20 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>116</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>128</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12491,20 +12647,20 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>328</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12512,20 +12668,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>2829</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>3032</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12533,20 +12689,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>419</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>441</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12554,20 +12710,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>32</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12575,19 +12731,19 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>85</v>
       </c>
     </row>
@@ -12596,20 +12752,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H112,'Social — theo ngày'!$A$6:$A$112,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$112,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>1385</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H113,'Social — theo ngày'!$A$6:$A$113,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$113,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>1437</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12651,7 +12807,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B70</f>
+        <f aca="false">'Social — 28 ngày'!B71</f>
         <v>116</v>
       </c>
     </row>
@@ -12672,8 +12828,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C70</f>
-        <v>171</v>
+        <f aca="false">'Social — 28 ngày'!C71</f>
+        <v>177</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12693,8 +12849,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D70</f>
-        <v>3957</v>
+        <f aca="false">'Social — 28 ngày'!D71</f>
+        <v>4026</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12714,8 +12870,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E70</f>
-        <v>499</v>
+        <f aca="false">'Social — 28 ngày'!E71</f>
+        <v>517</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12735,7 +12891,7 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F70</f>
+        <f aca="false">'Social — 28 ngày'!F71</f>
         <v>49</v>
       </c>
     </row>
@@ -12756,8 +12912,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G70</f>
-        <v>48</v>
+        <f aca="false">'Social — 28 ngày'!G71</f>
+        <v>57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12777,7 +12933,7 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H70</f>
+        <f aca="false">'Social — 28 ngày'!H71</f>
         <v>286</v>
       </c>
     </row>
@@ -12798,8 +12954,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I70</f>
-        <v>1767</v>
+        <f aca="false">'Social — 28 ngày'!I71</f>
+        <v>1790</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12819,8 +12975,8 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J70</f>
-        <v>139</v>
+        <f aca="false">'Social — 28 ngày'!J71</f>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12840,8 +12996,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K70</f>
-        <v>1263</v>
+        <f aca="false">'Social — 28 ngày'!K71</f>
+        <v>1250</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12861,7 +13017,7 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L70</f>
+        <f aca="false">'Social — 28 ngày'!L71</f>
         <v>80</v>
       </c>
     </row>
@@ -12882,8 +13038,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M70</f>
-        <v>38</v>
+        <f aca="false">'Social — 28 ngày'!M71</f>
+        <v>35</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12903,7 +13059,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N70</f>
+        <f aca="false">'Social — 28 ngày'!N71</f>
         <v>7</v>
       </c>
     </row>
@@ -12924,8 +13080,8 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O70</f>
-        <v>782</v>
+        <f aca="false">'Social — 28 ngày'!O71</f>
+        <v>783</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12974,8 +13130,8 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B70</f>
-        <v>19</v>
+        <f aca="false">SEO!B71</f>
+        <v>21</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12999,7 +13155,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C70</f>
+        <f aca="false">SEO!C71</f>
         <v>911</v>
       </c>
     </row>
@@ -13024,7 +13180,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D70</f>
+        <f aca="false">SEO!D71</f>
         <v>875</v>
       </c>
     </row>
@@ -13049,8 +13205,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E70</f>
-        <v>40.36</v>
+        <f aca="false">SEO!E71</f>
+        <v>39.58</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13074,8 +13230,8 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F70</f>
-        <v>9</v>
+        <f aca="false">SEO!F71</f>
+        <v>8</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13099,8 +13255,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G70</f>
-        <v>669</v>
+        <f aca="false">SEO!G71</f>
+        <v>672</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13124,8 +13280,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H70</f>
-        <v>419</v>
+        <f aca="false">SEO!H71</f>
+        <v>422</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13149,8 +13305,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I70</f>
-        <v>28</v>
+        <f aca="false">SEO!I71</f>
+        <v>29</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13174,8 +13330,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J70</f>
-        <v>2.8</v>
+        <f aca="false">SEO!J71</f>
+        <v>2.5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13199,8 +13355,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K70</f>
-        <v>1017</v>
+        <f aca="false">SEO!K71</f>
+        <v>1174</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13224,8 +13380,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L70</f>
-        <v>19.1</v>
+        <f aca="false">SEO!L71</f>
+        <v>18.3</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13249,8 +13405,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M70</f>
-        <v>110</v>
+        <f aca="false">SEO!M71</f>
+        <v>114</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13274,7 +13430,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N70</f>
+        <f aca="false">SEO!N71</f>
         <v>119</v>
       </c>
     </row>
@@ -13299,8 +13455,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O70</f>
-        <v>308</v>
+        <f aca="false">SEO!O71</f>
+        <v>311.2</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13342,7 +13498,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B67</f>
+        <f aca="false">Audit!B68</f>
         <v>93</v>
       </c>
     </row>
@@ -13363,7 +13519,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C67</f>
+        <f aca="false">Audit!C68</f>
         <v>98</v>
       </c>
     </row>
@@ -13384,7 +13540,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D67</f>
+        <f aca="false">Audit!D68</f>
         <v>97</v>
       </c>
     </row>
@@ -13405,7 +13561,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E67</f>
+        <f aca="false">Audit!E68</f>
         <v>93</v>
       </c>
     </row>
@@ -13426,7 +13582,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F67</f>
+        <f aca="false">Audit!F68</f>
         <v>118</v>
       </c>
     </row>
@@ -13447,7 +13603,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G67</f>
+        <f aca="false">Audit!G68</f>
         <v>98</v>
       </c>
     </row>
@@ -13468,7 +13624,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H67</f>
+        <f aca="false">Audit!H68</f>
         <v>119</v>
       </c>
     </row>
@@ -13489,7 +13645,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I67</f>
+        <f aca="false">Audit!I68</f>
         <v>98</v>
       </c>
     </row>
@@ -13510,8 +13666,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J67</f>
-        <v>308</v>
+        <f aca="false">Audit!J68</f>
+        <v>311.2</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13531,8 +13687,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K67</f>
-        <v>253</v>
+        <f aca="false">Audit!K68</f>
+        <v>255</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13552,8 +13708,8 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L67</f>
-        <v>242263</v>
+        <f aca="false">Audit!L68</f>
+        <v>243021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Social: index.html + dxl-metrics.xlsx 2026-10-26 re-run (LinkedIn read live)
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -7234,10 +7234,18 @@
       <c r="I73" s="16" t="n">
         <v>1933</v>
       </c>
-      <c r="J73" s="16"/>
-      <c r="K73" s="16"/>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
+      <c r="J73" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="K73" s="16" t="n">
+        <v>1275</v>
+      </c>
+      <c r="L73" s="16" t="n">
+        <v>82</v>
+      </c>
+      <c r="M73" s="16" t="n">
+        <v>38</v>
+      </c>
       <c r="N73" s="16" t="n">
         <v>7</v>
       </c>
@@ -13320,7 +13328,7 @@
       </c>
       <c r="E25" s="24" t="n">
         <f aca="false">'Social — 28 ngày'!J73</f>
-        <v>0</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13341,7 +13349,7 @@
       </c>
       <c r="E26" s="24" t="n">
         <f aca="false">'Social — 28 ngày'!K73</f>
-        <v>0</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13362,7 +13370,7 @@
       </c>
       <c r="E27" s="24" t="n">
         <f aca="false">'Social — 28 ngày'!L73</f>
-        <v>0</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13383,7 +13391,7 @@
       </c>
       <c r="E28" s="24" t="n">
         <f aca="false">'Social — 28 ngày'!M73</f>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Social: index.html 2026-10-29 + dxl-metrics.xlsx
</commit_message>
<xml_diff>
--- a/dxl-metrics.xlsx
+++ b/dxl-metrics.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">DX Living — dữ liệu báo cáo theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">Xuất ngày 2026-10-27 · nguồn: data/rollup.json của ba repo báo cáo</t>
+    <t xml:space="preserve">Xuất ngày 2026-10-29 · nguồn: data/rollup.json của ba repo báo cáo</t>
   </si>
   <si>
     <t xml:space="preserve">File này là gì</t>
@@ -96,31 +96,31 @@
     <t xml:space="preserve">Social — theo ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">114 dòng × 7 chỉ số · 2026-07-05 → 2026-10-26</t>
+    <t xml:space="preserve">115 dòng × 7 chỉ số · 2026-07-05 → 2026-10-27</t>
   </si>
   <si>
     <t xml:space="preserve">Social — 28 ngày</t>
   </si>
   <si>
-    <t xml:space="preserve">70 dòng × 14 chỉ số · 2026-07-23 → 2026-10-28</t>
+    <t xml:space="preserve">71 dòng × 14 chỉ số · 2026-07-23 → 2026-10-29</t>
   </si>
   <si>
     <t xml:space="preserve">SEO</t>
   </si>
   <si>
-    <t xml:space="preserve">70 dòng × 14 chỉ số · 2026-06-30 → 2026-10-28</t>
+    <t xml:space="preserve">71 dòng × 14 chỉ số · 2026-06-30 → 2026-10-29</t>
   </si>
   <si>
     <t xml:space="preserve">Audit</t>
   </si>
   <si>
-    <t xml:space="preserve">67 dòng × 11 chỉ số · 2026-07-27 → 2026-10-28</t>
+    <t xml:space="preserve">68 dòng × 11 chỉ số · 2026-07-27 → 2026-10-29</t>
   </si>
   <si>
     <t xml:space="preserve">Số theo NGÀY THẬT — cộng dồn được. Dựng lại từ chuỗi 28 giá trị trong mỗi file ngày, giữ lần đọc mới nhất cho mỗi ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 114 ngày · 7 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 115 ngày · 7 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">grain →</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">Ảnh chụp cửa sổ 28 ngày và chỉ số trạng thái — KHÔNG cộng dồn. Chỉ so đầu kỳ với cuối kỳ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 70 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Social/data/rollup.json · 71 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">FB — followers</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">GSC/GA4 là cửa sổ 28 ngày trượt; Ahrefs, TTFB, sitemap là trạng thái. KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 70 ngày · 14 chỉ số</t>
+    <t xml:space="preserve">Nguồn: SEO/data/rollup.json · 71 ngày · 14 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Ahrefs — trích dẫn AI</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Mỗi dòng là một lần crawl tại thời điểm. Điểm số và tốc độ — KHÔNG cộng dồn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 67 ngày · 11 chỉ số</t>
+    <t xml:space="preserve">Nguồn: Audit/data/rollup.json · 68 ngày · 11 chỉ số</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -981,7 +981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H119"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3991,6 +3991,30 @@
       <c r="G119" s="16"/>
       <c r="H119" s="16" t="n">
         <v>17</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="15" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B120" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C120" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="E120" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="F120" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G120" s="16"/>
+      <c r="H120" s="16" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4009,7 +4033,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7392,6 +7416,53 @@
         <v>7</v>
       </c>
       <c r="O75" s="16" t="n">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="15" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B76" s="16" t="n">
+        <v>117</v>
+      </c>
+      <c r="C76" s="16" t="n">
+        <v>167</v>
+      </c>
+      <c r="D76" s="16" t="n">
+        <v>4199</v>
+      </c>
+      <c r="E76" s="16" t="n">
+        <v>653</v>
+      </c>
+      <c r="F76" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="G76" s="16" t="n">
+        <v>66</v>
+      </c>
+      <c r="H76" s="16" t="n">
+        <v>337</v>
+      </c>
+      <c r="I76" s="16" t="n">
+        <v>1916</v>
+      </c>
+      <c r="J76" s="16" t="n">
+        <v>141</v>
+      </c>
+      <c r="K76" s="16" t="n">
+        <v>1268</v>
+      </c>
+      <c r="L76" s="16" t="n">
+        <v>82</v>
+      </c>
+      <c r="M76" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="N76" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O76" s="16" t="n">
         <v>869</v>
       </c>
     </row>
@@ -7411,7 +7482,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -10701,6 +10772,53 @@
       </c>
       <c r="O75" s="19" t="n">
         <v>318.4</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="15" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B76" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="C76" s="16" t="n">
+        <v>906</v>
+      </c>
+      <c r="D76" s="16" t="n">
+        <v>870</v>
+      </c>
+      <c r="E76" s="19" t="n">
+        <v>39.09</v>
+      </c>
+      <c r="F76" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G76" s="16" t="n">
+        <v>683</v>
+      </c>
+      <c r="H76" s="16" t="n">
+        <v>434</v>
+      </c>
+      <c r="I76" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="J76" s="19" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="K76" s="16" t="n">
+        <v>1580</v>
+      </c>
+      <c r="L76" s="19" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="M76" s="16" t="n">
+        <v>139</v>
+      </c>
+      <c r="N76" s="16" t="n">
+        <v>122</v>
+      </c>
+      <c r="O76" s="19" t="n">
+        <v>318.2</v>
       </c>
     </row>
   </sheetData>
@@ -10719,7 +10837,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -13222,6 +13340,44 @@
         <v>257</v>
       </c>
       <c r="L72" s="16" t="n">
+        <v>249426</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="15" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B73" s="16" t="n">
+        <v>94</v>
+      </c>
+      <c r="C73" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="D73" s="16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E73" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="F73" s="16" t="n">
+        <v>121</v>
+      </c>
+      <c r="G73" s="16" t="n">
+        <v>99</v>
+      </c>
+      <c r="H73" s="16" t="n">
+        <v>122</v>
+      </c>
+      <c r="I73" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="J73" s="19" t="n">
+        <v>318.2</v>
+      </c>
+      <c r="K73" s="16" t="n">
+        <v>258</v>
+      </c>
+      <c r="L73" s="16" t="n">
         <v>249426</v>
       </c>
     </row>
@@ -13290,19 +13446,19 @@
         <v>34</v>
       </c>
       <c r="B7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>125</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>195</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>160</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!B6:B119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!B6:B120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>152</v>
       </c>
     </row>
@@ -13311,19 +13467,19 @@
         <v>35</v>
       </c>
       <c r="B8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>106</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>147</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>354</v>
       </c>
       <c r="E8" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!C6:C119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!C6:C120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>433</v>
       </c>
     </row>
@@ -13332,20 +13488,20 @@
         <v>36</v>
       </c>
       <c r="B9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>3579</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>4978</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>4776</v>
       </c>
       <c r="E9" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!D6:D119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>3998</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!D6:D120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>4037</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13353,20 +13509,20 @@
         <v>37</v>
       </c>
       <c r="B10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>189</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>314</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>425</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!E6:E119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>606</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!E6:E120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>650</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13374,20 +13530,20 @@
         <v>38</v>
       </c>
       <c r="B11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>51</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>69</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>25</v>
       </c>
       <c r="E11" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!F6:F119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>63</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!F6:F120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>64</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13395,19 +13551,19 @@
         <v>39</v>
       </c>
       <c r="B12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>275</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>387</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>177</v>
       </c>
       <c r="E12" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!G6:G119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!G6:G120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
         <v>85</v>
       </c>
     </row>
@@ -13416,20 +13572,20 @@
         <v>40</v>
       </c>
       <c r="B13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,7,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,7,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,7,31))</f>
         <v>869</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,8,31))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,8,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,8,31))</f>
         <v>1161</v>
       </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,9,30))</f>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,9,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,9,30))</f>
         <v>2465</v>
       </c>
       <c r="E13" s="16" t="n">
-        <f aca="false">SUMIFS('Social — theo ngày'!H6:H119,'Social — theo ngày'!$A$6:$A$119,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$119,"&lt;="&amp;DATE(2026,10,31))</f>
-        <v>1761</v>
+        <f aca="false">SUMIFS('Social — theo ngày'!H6:H120,'Social — theo ngày'!$A$6:$A$120,"&gt;="&amp;DATE(2026,10,1),'Social — theo ngày'!$A$6:$A$120,"&lt;="&amp;DATE(2026,10,31))</f>
+        <v>1769</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13471,7 +13627,7 @@
         <v>116</v>
       </c>
       <c r="E17" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!B75</f>
+        <f aca="false">'Social — 28 ngày'!B76</f>
         <v>117</v>
       </c>
     </row>
@@ -13492,8 +13648,8 @@
         <v>141</v>
       </c>
       <c r="E18" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!C75</f>
-        <v>171</v>
+        <f aca="false">'Social — 28 ngày'!C76</f>
+        <v>167</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13513,8 +13669,8 @@
         <v>4519</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!D75</f>
-        <v>4255</v>
+        <f aca="false">'Social — 28 ngày'!D76</f>
+        <v>4199</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13534,8 +13690,8 @@
         <v>422</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!E75</f>
-        <v>609</v>
+        <f aca="false">'Social — 28 ngày'!E76</f>
+        <v>653</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13555,8 +13711,8 @@
         <v>49</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!F75</f>
-        <v>49</v>
+        <f aca="false">'Social — 28 ngày'!F76</f>
+        <v>50</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13576,8 +13732,8 @@
         <v>20</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!G75</f>
-        <v>68</v>
+        <f aca="false">'Social — 28 ngày'!G76</f>
+        <v>66</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13597,7 +13753,7 @@
         <v>87</v>
       </c>
       <c r="E23" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!H75</f>
+        <f aca="false">'Social — 28 ngày'!H76</f>
         <v>337</v>
       </c>
     </row>
@@ -13618,8 +13774,8 @@
         <v>2258</v>
       </c>
       <c r="E24" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!I75</f>
-        <v>1968</v>
+        <f aca="false">'Social — 28 ngày'!I76</f>
+        <v>1916</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13639,7 +13795,7 @@
         <v>102</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!J75</f>
+        <f aca="false">'Social — 28 ngày'!J76</f>
         <v>141</v>
       </c>
     </row>
@@ -13660,8 +13816,8 @@
         <v>1193</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!K75</f>
-        <v>1256</v>
+        <f aca="false">'Social — 28 ngày'!K76</f>
+        <v>1268</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13681,7 +13837,7 @@
         <v>24</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!L75</f>
+        <f aca="false">'Social — 28 ngày'!L76</f>
         <v>82</v>
       </c>
     </row>
@@ -13702,8 +13858,8 @@
         <v>36</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!M75</f>
-        <v>38</v>
+        <f aca="false">'Social — 28 ngày'!M76</f>
+        <v>39</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13723,7 +13879,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!N75</f>
+        <f aca="false">'Social — 28 ngày'!N76</f>
         <v>7</v>
       </c>
     </row>
@@ -13744,7 +13900,7 @@
         <v>634</v>
       </c>
       <c r="E30" s="24" t="n">
-        <f aca="false">'Social — 28 ngày'!O75</f>
+        <f aca="false">'Social — 28 ngày'!O76</f>
         <v>869</v>
       </c>
     </row>
@@ -13794,7 +13950,7 @@
         <v>16</v>
       </c>
       <c r="F34" s="24" t="n">
-        <f aca="false">SEO!B75</f>
+        <f aca="false">SEO!B76</f>
         <v>29</v>
       </c>
     </row>
@@ -13819,7 +13975,7 @@
         <v>918</v>
       </c>
       <c r="F35" s="24" t="n">
-        <f aca="false">SEO!C75</f>
+        <f aca="false">SEO!C76</f>
         <v>906</v>
       </c>
     </row>
@@ -13844,7 +14000,7 @@
         <v>882</v>
       </c>
       <c r="F36" s="24" t="n">
-        <f aca="false">SEO!D75</f>
+        <f aca="false">SEO!D76</f>
         <v>870</v>
       </c>
     </row>
@@ -13869,8 +14025,8 @@
         <v>33.99</v>
       </c>
       <c r="F37" s="24" t="n">
-        <f aca="false">SEO!E75</f>
-        <v>39.4</v>
+        <f aca="false">SEO!E76</f>
+        <v>39.09</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13894,8 +14050,8 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <f aca="false">SEO!F75</f>
-        <v>7</v>
+        <f aca="false">SEO!F76</f>
+        <v>4</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13919,8 +14075,8 @@
         <v>559</v>
       </c>
       <c r="F39" s="24" t="n">
-        <f aca="false">SEO!G75</f>
-        <v>698</v>
+        <f aca="false">SEO!G76</f>
+        <v>683</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13944,8 +14100,8 @@
         <v>394</v>
       </c>
       <c r="F40" s="24" t="n">
-        <f aca="false">SEO!H75</f>
-        <v>439</v>
+        <f aca="false">SEO!H76</f>
+        <v>434</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13969,8 +14125,8 @@
         <v>30</v>
       </c>
       <c r="F41" s="24" t="n">
-        <f aca="false">SEO!I75</f>
-        <v>22</v>
+        <f aca="false">SEO!I76</f>
+        <v>21</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13994,8 +14150,8 @@
         <v>2.8</v>
       </c>
       <c r="F42" s="24" t="n">
-        <f aca="false">SEO!J75</f>
-        <v>1.5</v>
+        <f aca="false">SEO!J76</f>
+        <v>1.3</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14019,8 +14175,8 @@
         <v>1056</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">SEO!K75</f>
-        <v>1501</v>
+        <f aca="false">SEO!K76</f>
+        <v>1580</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14044,8 +14200,8 @@
         <v>25.8</v>
       </c>
       <c r="F44" s="24" t="n">
-        <f aca="false">SEO!L75</f>
-        <v>20.9</v>
+        <f aca="false">SEO!L76</f>
+        <v>21.1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14069,8 +14225,8 @@
         <v>80</v>
       </c>
       <c r="F45" s="24" t="n">
-        <f aca="false">SEO!M75</f>
-        <v>138</v>
+        <f aca="false">SEO!M76</f>
+        <v>139</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14094,7 +14250,7 @@
         <v>119</v>
       </c>
       <c r="F46" s="24" t="n">
-        <f aca="false">SEO!N75</f>
+        <f aca="false">SEO!N76</f>
         <v>122</v>
       </c>
     </row>
@@ -14119,8 +14275,8 @@
         <v>342</v>
       </c>
       <c r="F47" s="24" t="n">
-        <f aca="false">SEO!O75</f>
-        <v>318.4</v>
+        <f aca="false">SEO!O76</f>
+        <v>318.2</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14162,7 +14318,7 @@
         <v>93</v>
       </c>
       <c r="E51" s="24" t="n">
-        <f aca="false">Audit!B72</f>
+        <f aca="false">Audit!B73</f>
         <v>94</v>
       </c>
     </row>
@@ -14183,7 +14339,7 @@
         <v>98</v>
       </c>
       <c r="E52" s="24" t="n">
-        <f aca="false">Audit!C72</f>
+        <f aca="false">Audit!C73</f>
         <v>98</v>
       </c>
     </row>
@@ -14204,7 +14360,7 @@
         <v>95</v>
       </c>
       <c r="E53" s="24" t="n">
-        <f aca="false">Audit!D72</f>
+        <f aca="false">Audit!D73</f>
         <v>97</v>
       </c>
     </row>
@@ -14225,7 +14381,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="24" t="n">
-        <f aca="false">Audit!E72</f>
+        <f aca="false">Audit!E73</f>
         <v>93</v>
       </c>
     </row>
@@ -14246,7 +14402,7 @@
         <v>118</v>
       </c>
       <c r="E55" s="24" t="n">
-        <f aca="false">Audit!F72</f>
+        <f aca="false">Audit!F73</f>
         <v>121</v>
       </c>
     </row>
@@ -14267,7 +14423,7 @@
         <v>98</v>
       </c>
       <c r="E56" s="24" t="n">
-        <f aca="false">Audit!G72</f>
+        <f aca="false">Audit!G73</f>
         <v>99</v>
       </c>
     </row>
@@ -14288,7 +14444,7 @@
         <v>119</v>
       </c>
       <c r="E57" s="24" t="n">
-        <f aca="false">Audit!H72</f>
+        <f aca="false">Audit!H73</f>
         <v>122</v>
       </c>
     </row>
@@ -14309,7 +14465,7 @@
         <v>92</v>
       </c>
       <c r="E58" s="24" t="n">
-        <f aca="false">Audit!I72</f>
+        <f aca="false">Audit!I73</f>
         <v>98</v>
       </c>
     </row>
@@ -14330,8 +14486,8 @@
         <v>342</v>
       </c>
       <c r="E59" s="24" t="n">
-        <f aca="false">Audit!J72</f>
-        <v>318.4</v>
+        <f aca="false">Audit!J73</f>
+        <v>318.2</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14351,8 +14507,8 @@
         <v>276</v>
       </c>
       <c r="E60" s="24" t="n">
-        <f aca="false">Audit!K72</f>
-        <v>257</v>
+        <f aca="false">Audit!K73</f>
+        <v>258</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14372,7 +14528,7 @@
         <v>241329</v>
       </c>
       <c r="E61" s="24" t="n">
-        <f aca="false">Audit!L72</f>
+        <f aca="false">Audit!L73</f>
         <v>249426</v>
       </c>
     </row>

</xml_diff>